<commit_message>
Gestion : onglet de coffrets Onsha proposés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6qThdJp8fvnL986bvjdNe
</commit_message>
<xml_diff>
--- a/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
+++ b/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Marges produits" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Simulateur commande" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Seuil de rentabilité" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Coffrets Onsha" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="386">
   <si>
     <t xml:space="preserve">Sunsoari · Tableau de marges et de gestion</t>
   </si>
@@ -1066,6 +1067,126 @@
   </si>
   <si>
     <t xml:space="preserve">Soit environ par semaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coffrets Onsha proposés · pour vendre les recharges par lot plutôt qu'à l'unité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propositions à tester, pas encore créées sur Shopify. Le prix proposé (bleu) est modifiable : tout se recalcule. Coûts et prix unitaires repris de l'onglet Marges produits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coffret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objectif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur si acheté à l'unité (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prix proposé TTC (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Économie cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coût de revient (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA hors TVA (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux de marge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il te reste si commandé seul (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparaison : il te reste avec 1 seule unité (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livraison offerte ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duo Filtres Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faire racheter 2 filtres au lieu d'1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 filtres thermaux Home au choix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rituel Saison Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recharge pour plusieurs mois, panier plus élevé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 filtres thermaux Home (au choix ou 1 de chaque senteur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trio Capsules Nomade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remplacer l'achat d'une capsule seule (en perte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 capsules thermales Nomade au choix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rituel Saison Nomade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recharge pour plusieurs mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 capsules thermales Nomade au choix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Douchette Habillée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendre la housse avec la douchette (housse seule en perte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 douchette filtrante + 1 housse au choix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duo Recharges Douchette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fidéliser les clientes de la douchette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 boîtes de 3 filtres sédiment (6 filtres)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set Découverte Home + 2 filtres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faire monter le panier dès le premier achat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set Découverte Home (coque + 4 filtres) + 2 filtres au choix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set Découverte Nomade + 3 capsules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set Découverte Nomade (coque + 4 capsules) + 3 capsules au choix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment lire : la colonne « Il te reste si commandé seul » compte le colis, l'emballage, le cadeau et la livraison payée par la cliente. Compare-la à la dernière colonne : c'est ce que tu gagnes en plus en vendant le lot plutôt qu'une seule unité.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Règle de prix utilisée : environ 7 à 16 % d'économie par rapport à l'unité. Assez pour donner envie, sans casser ta marge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le cadeau à 3 € pèse beaucoup sur les petits paniers : mets 0 dans Paramètres pour voir l'effet, ou réserve-le aux commandes à partir de 40 €.</t>
   </si>
 </sst>
 </file>
@@ -1791,6 +1912,550 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M16"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="27" t="s">
+        <v>348</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>349</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>350</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>351</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>354</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>355</v>
+      </c>
+      <c r="I4" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="J4" s="27" t="s">
+        <v>356</v>
+      </c>
+      <c r="K4" s="27" t="s">
+        <v>357</v>
+      </c>
+      <c r="L4" s="27" t="s">
+        <v>358</v>
+      </c>
+      <c r="M4" s="27" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="25" t="s">
+        <v>360</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="D5" s="35" t="n">
+        <f aca="false">2*'Marges produits'!$E$11</f>
+        <v>25.8</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="F5" s="36" t="n">
+        <f aca="false">IF(D5=0,0,1-E5/D5)</f>
+        <v>0.0736434108527133</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <f aca="false">2*'Marges produits'!$G$11</f>
+        <v>11.0006666666667</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E5/(1+Paramètres!$C$6),E5)</f>
+        <v>19.9166666666667</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <f aca="false">H5-G5-E5*Paramètres!$C$11-H5*Paramètres!$C$13</f>
+        <v>8.55750000000001</v>
+      </c>
+      <c r="J5" s="36" t="n">
+        <f aca="false">IF(H5=0,0,I5/H5)</f>
+        <v>0.429665271966527</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <f aca="false">I5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>3.6715</v>
+      </c>
+      <c r="L5" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$11</f>
+        <v>0.170166666666668</v>
+      </c>
+      <c r="M5" s="6" t="str">
+        <f aca="false">IF(E5&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="25" t="s">
+        <v>363</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="D6" s="35" t="n">
+        <f aca="false">4*'Marges produits'!$E$11</f>
+        <v>51.6</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="F6" s="36" t="n">
+        <f aca="false">IF(D6=0,0,1-E6/D6)</f>
+        <v>0.12984496124031</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <f aca="false">4*'Marges produits'!$G$11</f>
+        <v>22.0013333333333</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E6/(1+Paramètres!$C$6),E6)</f>
+        <v>37.4166666666667</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <f aca="false">H6-G6-E6*Paramètres!$C$11-H6*Paramètres!$C$13</f>
+        <v>14.7418333333333</v>
+      </c>
+      <c r="J6" s="36" t="n">
+        <f aca="false">IF(H6=0,0,I6/H6)</f>
+        <v>0.393991091314031</v>
+      </c>
+      <c r="K6" s="17" t="n">
+        <f aca="false">I6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>9.85583333333334</v>
+      </c>
+      <c r="L6" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$11</f>
+        <v>0.170166666666668</v>
+      </c>
+      <c r="M6" s="6" t="str">
+        <f aca="false">IF(E6&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="25" t="s">
+        <v>366</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D7" s="35" t="n">
+        <f aca="false">3*'Marges produits'!$E$13</f>
+        <v>20.7</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="F7" s="36" t="n">
+        <f aca="false">IF(D7=0,0,1-E7/D7)</f>
+        <v>0.135265700483092</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <f aca="false">3*'Marges produits'!$G$13</f>
+        <v>8.07495744680851</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E7/(1+Paramètres!$C$6),E7)</f>
+        <v>14.9166666666667</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <f aca="false">H7-G7-E7*Paramètres!$C$11-H7*Paramètres!$C$13</f>
+        <v>6.57320921985816</v>
+      </c>
+      <c r="J7" s="36" t="n">
+        <f aca="false">IF(H7=0,0,I7/H7)</f>
+        <v>0.440662070605016</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <f aca="false">I7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>1.68720921985816</v>
+      </c>
+      <c r="L7" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$13</f>
+        <v>-1.9311524822695</v>
+      </c>
+      <c r="M7" s="6" t="str">
+        <f aca="false">IF(E7&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>370</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="D8" s="35" t="n">
+        <f aca="false">6*'Marges produits'!$E$13</f>
+        <v>41.4</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F8" s="36" t="n">
+        <f aca="false">IF(D8=0,0,1-E8/D8)</f>
+        <v>0.157004830917875</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <f aca="false">6*'Marges produits'!$G$13</f>
+        <v>16.149914893617</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E8/(1+Paramètres!$C$6),E8)</f>
+        <v>29.0833333333333</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <f aca="false">H8-G8-E8*Paramètres!$C$11-H8*Paramètres!$C$13</f>
+        <v>12.4099184397163</v>
+      </c>
+      <c r="J8" s="36" t="n">
+        <f aca="false">IF(H8=0,0,I8/H8)</f>
+        <v>0.426702066695117</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <f aca="false">I8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>7.52391843971632</v>
+      </c>
+      <c r="L8" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$13</f>
+        <v>-1.9311524822695</v>
+      </c>
+      <c r="M8" s="6" t="str">
+        <f aca="false">IF(E8&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="25" t="s">
+        <v>372</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <f aca="false">1*'Marges produits'!$E$6+1*'Marges produits'!$E$8</f>
+        <v>33.8</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="F9" s="36" t="n">
+        <f aca="false">IF(D9=0,0,1-E9/D9)</f>
+        <v>0.115384615384615</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <f aca="false">1*'Marges produits'!$G$6+1*'Marges produits'!$G$8</f>
+        <v>11.9368936170213</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E9/(1+Paramètres!$C$6),E9)</f>
+        <v>24.9166666666667</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <f aca="false">H9-G9-E9*Paramètres!$C$11-H9*Paramètres!$C$13</f>
+        <v>12.5312730496454</v>
+      </c>
+      <c r="J9" s="36" t="n">
+        <f aca="false">IF(H9=0,0,I9/H9)</f>
+        <v>0.502927346474063</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <f aca="false">I9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>7.64527304964539</v>
+      </c>
+      <c r="L9" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$8</f>
+        <v>-1.11454964539007</v>
+      </c>
+      <c r="M9" s="6" t="str">
+        <f aca="false">IF(E9&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="25" t="s">
+        <v>375</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <f aca="false">2*'Marges produits'!$E$7</f>
+        <v>27.8</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F10" s="36" t="n">
+        <f aca="false">IF(D10=0,0,1-E10/D10)</f>
+        <v>0.10431654676259</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <f aca="false">2*'Marges produits'!$G$7</f>
+        <v>9.8303829787234</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E10/(1+Paramètres!$C$6),E10)</f>
+        <v>20.75</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <f aca="false">H10-G10-E10*Paramètres!$C$11-H10*Paramètres!$C$13</f>
+        <v>10.5461170212766</v>
+      </c>
+      <c r="J10" s="36" t="n">
+        <f aca="false">IF(H10=0,0,I10/H10)</f>
+        <v>0.508246603435017</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <f aca="false">I10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>5.6601170212766</v>
+      </c>
+      <c r="L10" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$7</f>
+        <v>1.57364184397163</v>
+      </c>
+      <c r="M10" s="6" t="str">
+        <f aca="false">IF(E10&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="25" t="s">
+        <v>378</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="D11" s="35" t="n">
+        <f aca="false">1*'Marges produits'!$E$16+2*'Marges produits'!$E$11</f>
+        <v>85.7</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>74.9</v>
+      </c>
+      <c r="F11" s="36" t="n">
+        <f aca="false">IF(D11=0,0,1-E11/D11)</f>
+        <v>0.126021003500583</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <f aca="false">1*'Marges produits'!$G$16+2*'Marges produits'!$G$11</f>
+        <v>34.4063404255319</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E11/(1+Paramètres!$C$6),E11)</f>
+        <v>62.4166666666667</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <f aca="false">H11-G11-E11*Paramètres!$C$11-H11*Paramètres!$C$13</f>
+        <v>26.8868262411348</v>
+      </c>
+      <c r="J11" s="36" t="n">
+        <f aca="false">IF(H11=0,0,I11/H11)</f>
+        <v>0.430763571286538</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <f aca="false">I11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>22.0008262411348</v>
+      </c>
+      <c r="L11" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$16</f>
+        <v>20.7264929078014</v>
+      </c>
+      <c r="M11" s="6" t="str">
+        <f aca="false">IF(E11&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="25" t="s">
+        <v>381</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <f aca="false">1*'Marges produits'!$E$17+3*'Marges produits'!$E$13</f>
+        <v>50.6</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="F12" s="36" t="n">
+        <f aca="false">IF(D12=0,0,1-E12/D12)</f>
+        <v>0.112648221343874</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <f aca="false">1*'Marges produits'!$G$17+3*'Marges produits'!$G$13</f>
+        <v>20.0118510638298</v>
+      </c>
+      <c r="H12" s="22" t="n">
+        <f aca="false">IF((Paramètres!$C$5="Assujettie"),E12/(1+Paramètres!$C$6),E12)</f>
+        <v>37.4166666666667</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <f aca="false">H12-G12-E12*Paramètres!$C$11-H12*Paramètres!$C$13</f>
+        <v>16.7313156028369</v>
+      </c>
+      <c r="J12" s="36" t="n">
+        <f aca="false">IF(H12=0,0,I12/H12)</f>
+        <v>0.447162109652656</v>
+      </c>
+      <c r="K12" s="17" t="n">
+        <f aca="false">I12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
+        <v>11.8453156028369</v>
+      </c>
+      <c r="L12" s="35" t="n">
+        <f aca="false">'Marges produits'!$N$17</f>
+        <v>7.6452730496454</v>
+      </c>
+      <c r="M12" s="6" t="str">
+        <f aca="false">IF(E12&gt;=Paramètres!$C$16,"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>383</v>
+      </c>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="32"/>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>384</v>
+      </c>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="32"/>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
+        <v>385</v>
+      </c>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32"/>
+      <c r="M16" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A16:M16"/>
+  </mergeCells>
+  <conditionalFormatting sqref="K5:K12">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>K5&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Gestion : fret réel Sullab (SUL-0413, EMS 773,61 $)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6qThdJp8fvnL986bvjdNe
</commit_message>
<xml_diff>
--- a/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
+++ b/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
@@ -265,7 +265,7 @@
     <t xml:space="preserve">Valeur de la marchandise (devise du fournisseur)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sullab : pro forma du 08/05/2026 (564 $). Shift : bon de commande (2 285 $). CNR : facture C-2026-0915 (435 €).</t>
+    <t xml:space="preserve">Sullab : facture commerciale SUL-0413 du 13/04/2026 (3 329 $, 492 pièces, 7 cartons, 85 kg). Shift : bon de commande (2 285 $). CNR : facture C-2026-0915 (435 €).</t>
   </si>
   <si>
     <t xml:space="preserve">Devise de la facture</t>
@@ -301,7 +301,7 @@
     <t xml:space="preserve">Fret international (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sullab et Shift : AUCUNE facture de transport reçue, ce sont des estimations à remplacer (facture EMS, DHL, FedEx ou du transitaire). CNR : 150 € facturés − 129,5 € pris en charge = 20,5 € (réel).</t>
+    <t xml:space="preserve">Sullab : RÉEL, 773,61 $ facturés sur SUL-0413 (reçu EMS de La Poste coréenne : 1 149 350 KRW pour 7 colis), soit 23 % de la marchandise. Shift : estimation à remplacer. CNR : 150 € facturés − 129,5 € pris en charge = 20,5 € (réel).</t>
   </si>
   <si>
     <t xml:space="preserve">Assurance transport (€)</t>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G5" s="35" t="n">
         <f aca="false">2*'Marges produits'!$G$11</f>
-        <v>11.0006666666667</v>
+        <v>10.1179030459597</v>
       </c>
       <c r="H5" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E5/(1+Paramètres!$C$6),E5)</f>
@@ -2015,19 +2015,19 @@
       </c>
       <c r="I5" s="17" t="n">
         <f aca="false">H5-G5-E5*Paramètres!$C$11-H5*Paramètres!$C$13</f>
-        <v>8.55750000000001</v>
+        <v>9.44026362070692</v>
       </c>
       <c r="J5" s="36" t="n">
         <f aca="false">IF(H5=0,0,I5/H5)</f>
-        <v>0.429665271966527</v>
+        <v>0.473988131583611</v>
       </c>
       <c r="K5" s="17" t="n">
         <f aca="false">I5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>3.6715</v>
+        <v>4.55426362070692</v>
       </c>
       <c r="L5" s="35" t="n">
         <f aca="false">'Marges produits'!$N$11</f>
-        <v>0.170166666666668</v>
+        <v>0.611548477020127</v>
       </c>
       <c r="M5" s="6" t="str">
         <f aca="false">IF(E5&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G6" s="35" t="n">
         <f aca="false">4*'Marges produits'!$G$11</f>
-        <v>22.0013333333333</v>
+        <v>20.2358060919195</v>
       </c>
       <c r="H6" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E6/(1+Paramètres!$C$6),E6)</f>
@@ -2065,19 +2065,19 @@
       </c>
       <c r="I6" s="17" t="n">
         <f aca="false">H6-G6-E6*Paramètres!$C$11-H6*Paramètres!$C$13</f>
-        <v>14.7418333333333</v>
+        <v>16.5073605747472</v>
       </c>
       <c r="J6" s="36" t="n">
         <f aca="false">IF(H6=0,0,I6/H6)</f>
-        <v>0.393991091314031</v>
+        <v>0.441176674603488</v>
       </c>
       <c r="K6" s="17" t="n">
         <f aca="false">I6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>9.85583333333334</v>
+        <v>11.6213605747472</v>
       </c>
       <c r="L6" s="35" t="n">
         <f aca="false">'Marges produits'!$N$11</f>
-        <v>0.170166666666668</v>
+        <v>0.611548477020127</v>
       </c>
       <c r="M6" s="6" t="str">
         <f aca="false">IF(E6&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="G7" s="35" t="n">
         <f aca="false">3*'Marges produits'!$G$13</f>
-        <v>8.07495744680851</v>
+        <v>7.42697138480024</v>
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E7/(1+Paramètres!$C$6),E7)</f>
@@ -2115,19 +2115,19 @@
       </c>
       <c r="I7" s="17" t="n">
         <f aca="false">H7-G7-E7*Paramètres!$C$11-H7*Paramètres!$C$13</f>
-        <v>6.57320921985816</v>
+        <v>7.22119528186643</v>
       </c>
       <c r="J7" s="36" t="n">
         <f aca="false">IF(H7=0,0,I7/H7)</f>
-        <v>0.440662070605016</v>
+        <v>0.484102476996632</v>
       </c>
       <c r="K7" s="17" t="n">
         <f aca="false">I7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>1.68720921985816</v>
+        <v>2.33519528186643</v>
       </c>
       <c r="L7" s="35" t="n">
         <f aca="false">'Marges produits'!$N$13</f>
-        <v>-1.9311524822695</v>
+        <v>-1.71515712826675</v>
       </c>
       <c r="M7" s="6" t="str">
         <f aca="false">IF(E7&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="G8" s="35" t="n">
         <f aca="false">6*'Marges produits'!$G$13</f>
-        <v>16.149914893617</v>
+        <v>14.8539427696005</v>
       </c>
       <c r="H8" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E8/(1+Paramètres!$C$6),E8)</f>
@@ -2165,19 +2165,19 @@
       </c>
       <c r="I8" s="17" t="n">
         <f aca="false">H8-G8-E8*Paramètres!$C$11-H8*Paramètres!$C$13</f>
-        <v>12.4099184397163</v>
+        <v>13.7058905637329</v>
       </c>
       <c r="J8" s="36" t="n">
         <f aca="false">IF(H8=0,0,I8/H8)</f>
-        <v>0.426702066695117</v>
+        <v>0.471262712793107</v>
       </c>
       <c r="K8" s="17" t="n">
         <f aca="false">I8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>7.52391843971632</v>
+        <v>8.81989056373286</v>
       </c>
       <c r="L8" s="35" t="n">
         <f aca="false">'Marges produits'!$N$13</f>
-        <v>-1.9311524822695</v>
+        <v>-1.71515712826675</v>
       </c>
       <c r="M8" s="6" t="str">
         <f aca="false">IF(E8&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="G9" s="35" t="n">
         <f aca="false">1*'Marges produits'!$G$6+1*'Marges produits'!$G$8</f>
-        <v>11.9368936170213</v>
+        <v>10.9790011775308</v>
       </c>
       <c r="H9" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E9/(1+Paramètres!$C$6),E9)</f>
@@ -2215,19 +2215,19 @@
       </c>
       <c r="I9" s="17" t="n">
         <f aca="false">H9-G9-E9*Paramètres!$C$11-H9*Paramètres!$C$13</f>
-        <v>12.5312730496454</v>
+        <v>13.4891654891359</v>
       </c>
       <c r="J9" s="36" t="n">
         <f aca="false">IF(H9=0,0,I9/H9)</f>
-        <v>0.502927346474063</v>
+        <v>0.541371190199433</v>
       </c>
       <c r="K9" s="17" t="n">
         <f aca="false">I9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>7.64527304964539</v>
+        <v>8.60316548913588</v>
       </c>
       <c r="L9" s="35" t="n">
         <f aca="false">'Marges produits'!$N$8</f>
-        <v>-1.11454964539007</v>
+        <v>-0.767078858516071</v>
       </c>
       <c r="M9" s="6" t="str">
         <f aca="false">IF(E9&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G10" s="35" t="n">
         <f aca="false">2*'Marges produits'!$G$7</f>
-        <v>9.8303829787234</v>
+        <v>9.04153038149594</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E10/(1+Paramètres!$C$6),E10)</f>
@@ -2265,19 +2265,19 @@
       </c>
       <c r="I10" s="17" t="n">
         <f aca="false">H10-G10-E10*Paramètres!$C$11-H10*Paramètres!$C$13</f>
-        <v>10.5461170212766</v>
+        <v>11.3349696185041</v>
       </c>
       <c r="J10" s="36" t="n">
         <f aca="false">IF(H10=0,0,I10/H10)</f>
-        <v>0.508246603435017</v>
+        <v>0.546263596072485</v>
       </c>
       <c r="K10" s="17" t="n">
         <f aca="false">I10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>5.6601170212766</v>
+        <v>6.44896961850406</v>
       </c>
       <c r="L10" s="35" t="n">
         <f aca="false">'Marges produits'!$N$7</f>
-        <v>1.57364184397163</v>
+        <v>1.96806814258536</v>
       </c>
       <c r="M10" s="6" t="str">
         <f aca="false">IF(E10&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="G11" s="35" t="n">
         <f aca="false">1*'Marges produits'!$G$16+2*'Marges produits'!$G$11</f>
-        <v>34.4063404255319</v>
+        <v>31.6453563352358</v>
       </c>
       <c r="H11" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E11/(1+Paramètres!$C$6),E11)</f>
@@ -2315,19 +2315,19 @@
       </c>
       <c r="I11" s="17" t="n">
         <f aca="false">H11-G11-E11*Paramètres!$C$11-H11*Paramètres!$C$13</f>
-        <v>26.8868262411348</v>
+        <v>29.6478103314309</v>
       </c>
       <c r="J11" s="36" t="n">
         <f aca="false">IF(H11=0,0,I11/H11)</f>
-        <v>0.430763571286538</v>
+        <v>0.474998296364714</v>
       </c>
       <c r="K11" s="17" t="n">
         <f aca="false">I11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>22.0008262411348</v>
+        <v>24.7618103314309</v>
       </c>
       <c r="L11" s="35" t="n">
         <f aca="false">'Marges produits'!$N$16</f>
-        <v>20.7264929078014</v>
+        <v>22.6047133773906</v>
       </c>
       <c r="M11" s="6" t="str">
         <f aca="false">IF(E11&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="G12" s="35" t="n">
         <f aca="false">1*'Marges produits'!$G$17+3*'Marges produits'!$G$13</f>
-        <v>20.0118510638298</v>
+        <v>18.405972562331</v>
       </c>
       <c r="H12" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E12/(1+Paramètres!$C$6),E12)</f>
@@ -2365,19 +2365,19 @@
       </c>
       <c r="I12" s="17" t="n">
         <f aca="false">H12-G12-E12*Paramètres!$C$11-H12*Paramètres!$C$13</f>
-        <v>16.7313156028369</v>
+        <v>18.3371941043356</v>
       </c>
       <c r="J12" s="36" t="n">
         <f aca="false">IF(H12=0,0,I12/H12)</f>
-        <v>0.447162109652656</v>
+        <v>0.490080911474449</v>
       </c>
       <c r="K12" s="17" t="n">
         <f aca="false">I12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>11.8453156028369</v>
+        <v>13.4511941043356</v>
       </c>
       <c r="L12" s="35" t="n">
         <f aca="false">'Marges produits'!$N$17</f>
-        <v>7.6452730496454</v>
+        <v>8.60316548913588</v>
       </c>
       <c r="M12" s="6" t="str">
         <f aca="false">IF(E12&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2796,12 +2796,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>564</v>
+        <v>3329</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>2285</v>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">C6*C9</f>
-        <v>485.04</v>
+        <v>2862.94</v>
       </c>
       <c r="D10" s="22" t="n">
         <f aca="false">D6*D9</f>
@@ -2889,8 +2889,9 @@
       <c r="B11" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>120</v>
+      <c r="C11" s="22" t="n">
+        <f aca="false">773.61*Paramètres!$C$7</f>
+        <v>665.3046</v>
       </c>
       <c r="D11" s="13" t="n">
         <v>250</v>
@@ -2999,7 +3000,7 @@
       </c>
       <c r="C17" s="22" t="n">
         <f aca="false">IF(C8="UE",0,(C10+C11+C12+C16)*Paramètres!$C$6)</f>
-        <v>121.008</v>
+        <v>705.64892</v>
       </c>
       <c r="D17" s="22" t="n">
         <f aca="false">IF(D8="UE",0,(D10+D11+D12+D16)*Paramètres!$C$6)</f>
@@ -3019,7 +3020,7 @@
       </c>
       <c r="C18" s="22" t="n">
         <f aca="false">SUM(C10:C14)+C16+C17</f>
-        <v>781.048</v>
+        <v>4288.89352</v>
       </c>
       <c r="D18" s="22" t="n">
         <f aca="false">SUM(D10:D14)+D16+D17</f>
@@ -3037,7 +3038,7 @@
       </c>
       <c r="C19" s="24" t="n">
         <f aca="false">IF(C10=0,1,(C18-C17)/C10)</f>
-        <v>1.36079498598054</v>
+        <v>1.25159612146954</v>
       </c>
       <c r="D19" s="24" t="n">
         <f aca="false">IF(D10=0,1,(D18-D17)/D10)</f>
@@ -3057,7 +3058,7 @@
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">IF(C10=0,1,C18/C10)</f>
-        <v>1.61027544120073</v>
+        <v>1.4980731415957</v>
       </c>
       <c r="D20" s="24" t="n">
         <f aca="false">IF(D10=0,1,D18/D10)</f>
@@ -3077,7 +3078,7 @@
       </c>
       <c r="C21" s="26" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),C19,C20)</f>
-        <v>1.36079498598054</v>
+        <v>1.25159612146954</v>
       </c>
       <c r="D21" s="26" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),D19,D20)</f>
@@ -3240,7 +3241,7 @@
       </c>
       <c r="O5" s="17" t="n">
         <f aca="false">N5*Import!$C$21</f>
-        <v>7.6068439716312</v>
+        <v>6.99642231901472</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3290,7 +3291,7 @@
       </c>
       <c r="O6" s="17" t="n">
         <f aca="false">N6*Import!$C$21</f>
-        <v>4.33004964539007</v>
+        <v>3.98257885851607</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3342,7 +3343,7 @@
       </c>
       <c r="O7" s="17" t="n">
         <f aca="false">N7*Import!$C$21</f>
-        <v>4.9151914893617</v>
+        <v>4.52076519074797</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3394,7 +3395,7 @@
       </c>
       <c r="O8" s="17" t="n">
         <f aca="false">N8*Import!$C$21</f>
-        <v>7.02170212765957</v>
+        <v>6.45823598678282</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3446,7 +3447,7 @@
       </c>
       <c r="O9" s="17" t="n">
         <f aca="false">N9*Import!$C$21</f>
-        <v>7.6068439716312</v>
+        <v>6.99642231901472</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3496,7 +3497,7 @@
       </c>
       <c r="O10" s="17" t="n">
         <f aca="false">N10*Import!$C$21</f>
-        <v>11.9368936170213</v>
+        <v>10.9790011775308</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3546,7 +3547,7 @@
       </c>
       <c r="O11" s="17" t="n">
         <f aca="false">N11*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3596,7 +3597,7 @@
       </c>
       <c r="O12" s="17" t="n">
         <f aca="false">N12*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3646,7 +3647,7 @@
       </c>
       <c r="O13" s="17" t="n">
         <f aca="false">N13*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3696,7 +3697,7 @@
       </c>
       <c r="O14" s="17" t="n">
         <f aca="false">N14*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3746,7 +3747,7 @@
       </c>
       <c r="O15" s="17" t="n">
         <f aca="false">N15*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3796,7 +3797,7 @@
       </c>
       <c r="O16" s="17" t="n">
         <f aca="false">N16*Import!$C$21</f>
-        <v>7.25575886524823</v>
+        <v>6.67351051967558</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3846,7 +3847,7 @@
       </c>
       <c r="O17" s="17" t="n">
         <f aca="false">N17*Import!$C$21</f>
-        <v>23.4056737588652</v>
+        <v>21.5274532892761</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3896,7 +3897,7 @@
       </c>
       <c r="O18" s="17" t="n">
         <f aca="false">N18*Import!$C$21</f>
-        <v>5.50033333333333</v>
+        <v>5.05895152297987</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3946,7 +3947,7 @@
       </c>
       <c r="O19" s="17" t="n">
         <f aca="false">N19*Import!$C$21</f>
-        <v>5.50033333333333</v>
+        <v>5.05895152297987</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3996,7 +3997,7 @@
       </c>
       <c r="O20" s="17" t="n">
         <f aca="false">N20*Import!$C$21</f>
-        <v>5.50033333333333</v>
+        <v>5.05895152297987</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4046,7 +4047,7 @@
       </c>
       <c r="O21" s="17" t="n">
         <f aca="false">N21*Import!$C$21</f>
-        <v>5.50033333333333</v>
+        <v>5.05895152297987</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4096,7 +4097,7 @@
       </c>
       <c r="O22" s="17" t="n">
         <f aca="false">N22*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4148,7 +4149,7 @@
       </c>
       <c r="O23" s="17" t="n">
         <f aca="false">N23*Import!$C$21</f>
-        <v>6.31953191489362</v>
+        <v>5.81241238810454</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4200,7 +4201,7 @@
       </c>
       <c r="O24" s="17" t="n">
         <f aca="false">N24*Import!$C$21</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
     </row>
   </sheetData>
@@ -4988,7 +4989,7 @@
       </c>
       <c r="G5" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$16</f>
-        <v>7.25575886524823</v>
+        <v>6.67351051967558</v>
       </c>
       <c r="H5" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E5/(1+Paramètres!$C$6),E5)</f>
@@ -5004,23 +5005,23 @@
       </c>
       <c r="K5" s="17" t="n">
         <f aca="false">IF(G5=0,0,H5-G5-I5-J5)</f>
-        <v>12.3024078014184</v>
+        <v>12.8846561469911</v>
       </c>
       <c r="L5" s="36" t="n">
         <f aca="false">IF(H5=0,0,K5/H5)</f>
-        <v>0.61769411555239</v>
+        <v>0.646928342108339</v>
       </c>
       <c r="M5" s="33" t="n">
         <f aca="false">IF(G5=0,0,E5/G5)</f>
-        <v>3.29393526492041</v>
+        <v>3.58132349226624</v>
       </c>
       <c r="N5" s="17" t="n">
         <f aca="false">IF(G5=0,0,K5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>7.41640780141844</v>
+        <v>7.99865614699109</v>
       </c>
       <c r="O5" s="22" t="n">
         <f aca="false">G5*Paramètres!$C$25</f>
-        <v>21.7672765957447</v>
+        <v>20.0205315590267</v>
       </c>
       <c r="P5" s="6" t="str">
         <f aca="false">IF(G5=0,"Prix fournisseur manquant",IF(N5&lt;0,"Perte si vendu seul",IF(L5&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5049,7 +5050,7 @@
       </c>
       <c r="G6" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$5</f>
-        <v>7.6068439716312</v>
+        <v>6.99642231901472</v>
       </c>
       <c r="H6" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E6/(1+Paramètres!$C$6),E6)</f>
@@ -5065,23 +5066,23 @@
       </c>
       <c r="K6" s="17" t="n">
         <f aca="false">IF(G6=0,0,H6-G6-I6-J6)</f>
-        <v>11.9513226950355</v>
+        <v>12.561744347652</v>
       </c>
       <c r="L6" s="36" t="n">
         <f aca="false">IF(H6=0,0,K6/H6)</f>
-        <v>0.600066411466216</v>
+        <v>0.630715197371646</v>
       </c>
       <c r="M6" s="33" t="n">
         <f aca="false">IF(G6=0,0,E6/G6)</f>
-        <v>3.14190748346254</v>
+        <v>3.41603163877703</v>
       </c>
       <c r="N6" s="17" t="n">
         <f aca="false">IF(G6=0,0,K6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>7.06532269503547</v>
+        <v>7.67574434765195</v>
       </c>
       <c r="O6" s="22" t="n">
         <f aca="false">G6*Paramètres!$C$25</f>
-        <v>22.8205319148936</v>
+        <v>20.9892669570442</v>
       </c>
       <c r="P6" s="6" t="str">
         <f aca="false">IF(G6=0,"Prix fournisseur manquant",IF(N6&lt;0,"Perte si vendu seul",IF(L6&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5110,7 +5111,7 @@
       </c>
       <c r="G7" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$7</f>
-        <v>4.9151914893617</v>
+        <v>4.52076519074797</v>
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E7/(1+Paramètres!$C$6),E7)</f>
@@ -5126,23 +5127,23 @@
       </c>
       <c r="K7" s="17" t="n">
         <f aca="false">IF(G7=0,0,H7-G7-I7-J7)</f>
-        <v>6.45964184397163</v>
+        <v>6.85406814258536</v>
       </c>
       <c r="L7" s="36" t="n">
         <f aca="false">IF(H7=0,0,K7/H7)</f>
-        <v>0.557666921781724</v>
+        <v>0.591718113028952</v>
       </c>
       <c r="M7" s="33" t="n">
         <f aca="false">IF(G7=0,0,E7/G7)</f>
-        <v>2.82796713619088</v>
+        <v>3.07470072288807</v>
       </c>
       <c r="N7" s="17" t="n">
         <f aca="false">IF(G7=0,0,K7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>1.57364184397163</v>
+        <v>1.96806814258536</v>
       </c>
       <c r="O7" s="22" t="n">
         <f aca="false">G7*Paramètres!$C$25</f>
-        <v>14.7455744680851</v>
+        <v>13.5622955722439</v>
       </c>
       <c r="P7" s="6" t="str">
         <f aca="false">IF(G7=0,"Prix fournisseur manquant",IF(N7&lt;0,"Perte si vendu seul",IF(L7&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5171,7 +5172,7 @@
       </c>
       <c r="G8" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$6</f>
-        <v>4.33004964539007</v>
+        <v>3.98257885851607</v>
       </c>
       <c r="H8" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E8/(1+Paramètres!$C$6),E8)</f>
@@ -5187,23 +5188,23 @@
       </c>
       <c r="K8" s="17" t="n">
         <f aca="false">IF(G8=0,0,H8-G8-I8-J8)</f>
-        <v>3.77145035460993</v>
+        <v>4.11892114148393</v>
       </c>
       <c r="L8" s="36" t="n">
         <f aca="false">IF(H8=0,0,K8/H8)</f>
-        <v>0.457145497528476</v>
+        <v>0.499263168664719</v>
       </c>
       <c r="M8" s="33" t="n">
         <f aca="false">IF(G8=0,0,E8/G8)</f>
-        <v>2.28634791994588</v>
+        <v>2.48582648371934</v>
       </c>
       <c r="N8" s="17" t="n">
         <f aca="false">IF(G8=0,0,K8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>-1.11454964539007</v>
+        <v>-0.767078858516071</v>
       </c>
       <c r="O8" s="22" t="n">
         <f aca="false">G8*Paramètres!$C$25</f>
-        <v>12.9901489361702</v>
+        <v>11.9477365755482</v>
       </c>
       <c r="P8" s="6" t="str">
         <f aca="false">IF(G8=0,"Prix fournisseur manquant",IF(N8&lt;0,"Perte si vendu seul",IF(L8&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5232,7 +5233,7 @@
       </c>
       <c r="G9" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$22</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
       <c r="H9" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E9/(1+Paramètres!$C$6),E9)</f>
@@ -5248,23 +5249,23 @@
       </c>
       <c r="K9" s="17" t="n">
         <f aca="false">IF(G9=0,0,H9-G9-I9-J9)</f>
-        <v>13.5931808510638</v>
+        <v>13.8091762050666</v>
       </c>
       <c r="L9" s="36" t="n">
         <f aca="false">IF(H9=0,0,K9/H9)</f>
-        <v>0.819689297551588</v>
+        <v>0.832714143019091</v>
       </c>
       <c r="M9" s="33" t="n">
         <f aca="false">IF(G9=0,0,E9/G9)</f>
-        <v>7.39322781491504</v>
+        <v>8.03826982855754</v>
       </c>
       <c r="N9" s="17" t="n">
         <f aca="false">IF(G9=0,0,K9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>8.70718085106383</v>
+        <v>8.92317620506659</v>
       </c>
       <c r="O9" s="22" t="n">
         <f aca="false">G9*Paramètres!$C$25</f>
-        <v>8.07495744680851</v>
+        <v>7.42697138480024</v>
       </c>
       <c r="P9" s="6" t="str">
         <f aca="false">IF(G9=0,"Prix fournisseur manquant",IF(N9&lt;0,"Perte si vendu seul",IF(L9&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5293,7 +5294,7 @@
       </c>
       <c r="G10" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$15</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E10/(1+Paramètres!$C$6),E10)</f>
@@ -5309,23 +5310,23 @@
       </c>
       <c r="K10" s="17" t="n">
         <f aca="false">IF(G10=0,0,H10-G10-I10-J10)</f>
-        <v>5.4098475177305</v>
+        <v>5.62584287173325</v>
       </c>
       <c r="L10" s="36" t="n">
         <f aca="false">IF(H10=0,0,K10/H10)</f>
-        <v>0.655739093058242</v>
+        <v>0.681920348088879</v>
       </c>
       <c r="M10" s="33" t="n">
         <f aca="false">IF(G10=0,0,E10/G10)</f>
-        <v>3.67803795817381</v>
+        <v>3.99893825641808</v>
       </c>
       <c r="N10" s="17" t="n">
         <f aca="false">IF(G10=0,0,K10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>0.523847517730497</v>
+        <v>0.739842871733253</v>
       </c>
       <c r="O10" s="22" t="n">
         <f aca="false">G10*Paramètres!$C$25</f>
-        <v>8.07495744680851</v>
+        <v>7.42697138480024</v>
       </c>
       <c r="P10" s="6" t="str">
         <f aca="false">IF(G10=0,"Prix fournisseur manquant",IF(N10&lt;0,"Perte si vendu seul",IF(L10&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5354,7 +5355,7 @@
       </c>
       <c r="G11" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$18</f>
-        <v>5.50033333333333</v>
+        <v>5.05895152297987</v>
       </c>
       <c r="H11" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E11/(1+Paramètres!$C$6),E11)</f>
@@ -5370,23 +5371,23 @@
       </c>
       <c r="K11" s="17" t="n">
         <f aca="false">IF(G11=0,0,H11-G11-I11-J11)</f>
-        <v>5.05616666666667</v>
+        <v>5.49754847702013</v>
       </c>
       <c r="L11" s="36" t="n">
         <f aca="false">IF(H11=0,0,K11/H11)</f>
-        <v>0.470341085271318</v>
+        <v>0.511399858327454</v>
       </c>
       <c r="M11" s="33" t="n">
         <f aca="false">IF(G11=0,0,E11/G11)</f>
-        <v>2.34531240530877</v>
+        <v>2.54993548394421</v>
       </c>
       <c r="N11" s="17" t="n">
         <f aca="false">IF(G11=0,0,K11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>0.170166666666668</v>
+        <v>0.611548477020127</v>
       </c>
       <c r="O11" s="22" t="n">
         <f aca="false">G11*Paramètres!$C$25</f>
-        <v>16.501</v>
+        <v>15.1768545689396</v>
       </c>
       <c r="P11" s="6" t="str">
         <f aca="false">IF(G11=0,"Prix fournisseur manquant",IF(N11&lt;0,"Perte si vendu seul",IF(L11&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5415,7 +5416,7 @@
       </c>
       <c r="G12" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$18</f>
-        <v>5.50033333333333</v>
+        <v>5.05895152297987</v>
       </c>
       <c r="H12" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E12/(1+Paramètres!$C$6),E12)</f>
@@ -5431,23 +5432,23 @@
       </c>
       <c r="K12" s="17" t="n">
         <f aca="false">IF(G12=0,0,H12-G12-I12-J12)</f>
-        <v>5.05616666666667</v>
+        <v>5.49754847702013</v>
       </c>
       <c r="L12" s="36" t="n">
         <f aca="false">IF(H12=0,0,K12/H12)</f>
-        <v>0.470341085271318</v>
+        <v>0.511399858327454</v>
       </c>
       <c r="M12" s="33" t="n">
         <f aca="false">IF(G12=0,0,E12/G12)</f>
-        <v>2.34531240530877</v>
+        <v>2.54993548394421</v>
       </c>
       <c r="N12" s="17" t="n">
         <f aca="false">IF(G12=0,0,K12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>0.170166666666668</v>
+        <v>0.611548477020127</v>
       </c>
       <c r="O12" s="22" t="n">
         <f aca="false">G12*Paramètres!$C$25</f>
-        <v>16.501</v>
+        <v>15.1768545689396</v>
       </c>
       <c r="P12" s="6" t="str">
         <f aca="false">IF(G12=0,"Prix fournisseur manquant",IF(N12&lt;0,"Perte si vendu seul",IF(L12&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5476,7 +5477,7 @@
       </c>
       <c r="G13" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$11</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
       <c r="H13" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E13/(1+Paramètres!$C$6),E13)</f>
@@ -5492,23 +5493,23 @@
       </c>
       <c r="K13" s="17" t="n">
         <f aca="false">IF(G13=0,0,H13-G13-I13-J13)</f>
-        <v>2.9548475177305</v>
+        <v>3.17084287173326</v>
       </c>
       <c r="L13" s="36" t="n">
         <f aca="false">IF(H13=0,0,K13/H13)</f>
-        <v>0.513886524822695</v>
+        <v>0.551450934214479</v>
       </c>
       <c r="M13" s="33" t="n">
         <f aca="false">IF(G13=0,0,E13/G13)</f>
-        <v>2.56348100115145</v>
+        <v>2.78713878477623</v>
       </c>
       <c r="N13" s="17" t="n">
         <f aca="false">IF(G13=0,0,K13-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E13&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>-1.9311524822695</v>
+        <v>-1.71515712826675</v>
       </c>
       <c r="O13" s="22" t="n">
         <f aca="false">G13*Paramètres!$C$25</f>
-        <v>8.07495744680851</v>
+        <v>7.42697138480024</v>
       </c>
       <c r="P13" s="6" t="str">
         <f aca="false">IF(G13=0,"Prix fournisseur manquant",IF(N13&lt;0,"Perte si vendu seul",IF(L13&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5537,7 +5538,7 @@
       </c>
       <c r="G14" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$22+'Tarifs Onsha-Sullab'!$O$18</f>
-        <v>8.19198581560283</v>
+        <v>7.53460865124662</v>
       </c>
       <c r="H14" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E14/(1+Paramètres!$C$6),E14)</f>
@@ -5553,23 +5554,23 @@
       </c>
       <c r="K14" s="17" t="n">
         <f aca="false">IF(G14=0,0,H14-G14-I14-J14)</f>
-        <v>16.2761808510638</v>
+        <v>16.9335580154201</v>
       </c>
       <c r="L14" s="36" t="n">
         <f aca="false">IF(H14=0,0,K14/H14)</f>
-        <v>0.653224649541023</v>
+        <v>0.679607679548631</v>
       </c>
       <c r="M14" s="33" t="n">
         <f aca="false">IF(G14=0,0,E14/G14)</f>
-        <v>3.6499086635442</v>
+        <v>3.9683547459433</v>
       </c>
       <c r="N14" s="17" t="n">
         <f aca="false">IF(G14=0,0,K14-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E14&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>11.3901808510638</v>
+        <v>12.0475580154201</v>
       </c>
       <c r="O14" s="22" t="n">
         <f aca="false">G14*Paramètres!$C$25</f>
-        <v>24.5759574468085</v>
+        <v>22.6038259537399</v>
       </c>
       <c r="P14" s="6" t="str">
         <f aca="false">IF(G14=0,"Prix fournisseur manquant",IF(N14&lt;0,"Perte si vendu seul",IF(L14&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5598,7 +5599,7 @@
       </c>
       <c r="G15" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$16+'Tarifs Onsha-Sullab'!$O$22+'Tarifs Onsha-Sullab'!$O$18</f>
-        <v>15.4477446808511</v>
+        <v>14.2081191709222</v>
       </c>
       <c r="H15" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E15/(1+Paramètres!$C$6),E15)</f>
@@ -5614,23 +5615,23 @@
       </c>
       <c r="K15" s="17" t="n">
         <f aca="false">IF(G15=0,0,H15-G15-I15-J15)</f>
-        <v>25.3870886524823</v>
+        <v>26.6267141624111</v>
       </c>
       <c r="L15" s="36" t="n">
         <f aca="false">IF(H15=0,0,K15/H15)</f>
-        <v>0.610511149959494</v>
+        <v>0.640321783464797</v>
       </c>
       <c r="M15" s="33" t="n">
         <f aca="false">IF(G15=0,0,E15/G15)</f>
-        <v>3.23024499892569</v>
+        <v>3.51207639798823</v>
       </c>
       <c r="N15" s="17" t="n">
         <f aca="false">IF(G15=0,0,K15-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E15&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>20.5010886524823</v>
+        <v>21.7407141624111</v>
       </c>
       <c r="O15" s="22" t="n">
         <f aca="false">G15*Paramètres!$C$25</f>
-        <v>46.3432340425532</v>
+        <v>42.6243575127666</v>
       </c>
       <c r="P15" s="6" t="str">
         <f aca="false">IF(G15=0,"Prix fournisseur manquant",IF(N15&lt;0,"Perte si vendu seul",IF(L15&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5659,7 +5660,7 @@
       </c>
       <c r="G16" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$17</f>
-        <v>23.4056737588652</v>
+        <v>21.5274532892761</v>
       </c>
       <c r="H16" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E16/(1+Paramètres!$C$6),E16)</f>
@@ -5675,23 +5676,23 @@
       </c>
       <c r="K16" s="17" t="n">
         <f aca="false">IF(G16=0,0,H16-G16-I16-J16)</f>
-        <v>25.6124929078014</v>
+        <v>27.4907133773906</v>
       </c>
       <c r="L16" s="36" t="n">
         <f aca="false">IF(H16=0,0,K16/H16)</f>
-        <v>0.513105033211381</v>
+        <v>0.550732154471932</v>
       </c>
       <c r="M16" s="33" t="n">
         <f aca="false">IF(G16=0,0,E16/G16)</f>
-        <v>2.55920853281619</v>
+        <v>2.78249355346827</v>
       </c>
       <c r="N16" s="17" t="n">
         <f aca="false">IF(G16=0,0,K16-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E16&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>20.7264929078014</v>
+        <v>22.6047133773906</v>
       </c>
       <c r="O16" s="22" t="n">
         <f aca="false">G16*Paramètres!$C$25</f>
-        <v>70.2170212765957</v>
+        <v>64.5823598678282</v>
       </c>
       <c r="P16" s="6" t="str">
         <f aca="false">IF(G16=0,"Prix fournisseur manquant",IF(N16&lt;0,"Perte si vendu seul",IF(L16&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5720,7 +5721,7 @@
       </c>
       <c r="G17" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$10</f>
-        <v>11.9368936170213</v>
+        <v>10.9790011775308</v>
       </c>
       <c r="H17" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E17/(1+Paramètres!$C$6),E17)</f>
@@ -5736,23 +5737,23 @@
       </c>
       <c r="K17" s="17" t="n">
         <f aca="false">IF(G17=0,0,H17-G17-I17-J17)</f>
-        <v>12.5312730496454</v>
+        <v>13.4891654891359</v>
       </c>
       <c r="L17" s="36" t="n">
         <f aca="false">IF(H17=0,0,K17/H17)</f>
-        <v>0.502927346474063</v>
+        <v>0.541371190199433</v>
       </c>
       <c r="M17" s="33" t="n">
         <f aca="false">IF(G17=0,0,E17/G17)</f>
-        <v>2.50483927890288</v>
+        <v>2.72338070800031</v>
       </c>
       <c r="N17" s="17" t="n">
         <f aca="false">IF(G17=0,0,K17-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E17&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>7.6452730496454</v>
+        <v>8.60316548913588</v>
       </c>
       <c r="O17" s="22" t="n">
         <f aca="false">G17*Paramètres!$C$25</f>
-        <v>35.8106808510638</v>
+        <v>32.9370035325924</v>
       </c>
       <c r="P17" s="6" t="str">
         <f aca="false">IF(G17=0,"Prix fournisseur manquant",IF(N17&lt;0,"Perte si vendu seul",IF(L17&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5781,7 +5782,7 @@
       </c>
       <c r="G18" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$16+'Tarifs Onsha-Sullab'!$O$17</f>
-        <v>30.6614326241135</v>
+        <v>28.2009638089516</v>
       </c>
       <c r="H18" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E18/(1+Paramètres!$C$6),E18)</f>
@@ -5797,23 +5798,23 @@
       </c>
       <c r="K18" s="17" t="n">
         <f aca="false">IF(G18=0,0,H18-G18-I18-J18)</f>
-        <v>34.7234007092199</v>
+        <v>37.1838695243817</v>
       </c>
       <c r="L18" s="36" t="n">
         <f aca="false">IF(H18=0,0,K18/H18)</f>
-        <v>0.52150288924986</v>
+        <v>0.558456113006984</v>
       </c>
       <c r="M18" s="33" t="n">
         <f aca="false">IF(G18=0,0,E18/G18)</f>
-        <v>2.60587954188296</v>
+        <v>2.83323650004607</v>
       </c>
       <c r="N18" s="17" t="n">
         <f aca="false">IF(G18=0,0,K18-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E18&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>29.8374007092199</v>
+        <v>32.2978695243817</v>
       </c>
       <c r="O18" s="22" t="n">
         <f aca="false">G18*Paramètres!$C$25</f>
-        <v>91.9842978723404</v>
+        <v>84.6028914268549</v>
       </c>
       <c r="P18" s="6" t="str">
         <f aca="false">IF(G18=0,"Prix fournisseur manquant",IF(N18&lt;0,"Perte si vendu seul",IF(L18&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5842,7 +5843,7 @@
       </c>
       <c r="G19" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$5+'Tarifs Onsha-Sullab'!$O$7+'Tarifs Onsha-Sullab'!$O$10</f>
-        <v>24.4589290780142</v>
+        <v>22.4961886872935</v>
       </c>
       <c r="H19" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E19/(1+Paramètres!$C$6),E19)</f>
@@ -5858,23 +5859,23 @@
       </c>
       <c r="K19" s="17" t="n">
         <f aca="false">IF(G19=0,0,H19-G19-I19-J19)</f>
-        <v>24.5592375886525</v>
+        <v>26.5219779793732</v>
       </c>
       <c r="L19" s="36" t="n">
         <f aca="false">IF(H19=0,0,K19/H19)</f>
-        <v>0.492004759705893</v>
+        <v>0.531325101423169</v>
       </c>
       <c r="M19" s="33" t="n">
         <f aca="false">IF(G19=0,0,E19/G19)</f>
-        <v>2.44900338068535</v>
+        <v>2.66267325690744</v>
       </c>
       <c r="N19" s="17" t="n">
         <f aca="false">IF(G19=0,0,K19-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E19&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>19.6732375886525</v>
+        <v>21.6359779793732</v>
       </c>
       <c r="O19" s="22" t="n">
         <f aca="false">G19*Paramètres!$C$25</f>
-        <v>73.3767872340425</v>
+        <v>67.4885660618804</v>
       </c>
       <c r="P19" s="6" t="str">
         <f aca="false">IF(G19=0,"Prix fournisseur manquant",IF(N19&lt;0,"Perte si vendu seul",IF(L19&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5903,7 +5904,7 @@
       </c>
       <c r="G20" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$23</f>
-        <v>6.31953191489362</v>
+        <v>5.81241238810454</v>
       </c>
       <c r="H20" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E20/(1+Paramètres!$C$6),E20)</f>
@@ -5919,23 +5920,23 @@
       </c>
       <c r="K20" s="17" t="n">
         <f aca="false">IF(G20=0,0,H20-G20-I20-J20)</f>
-        <v>14.8753014184397</v>
+        <v>15.3824209452288</v>
       </c>
       <c r="L20" s="36" t="n">
         <f aca="false">IF(H20=0,0,K20/H20)</f>
-        <v>0.689203154522303</v>
+        <v>0.712699039933381</v>
       </c>
       <c r="M20" s="33" t="n">
         <f aca="false">IF(G20=0,0,E20/G20)</f>
-        <v>4.09840481048287</v>
+        <v>4.455981143562</v>
       </c>
       <c r="N20" s="17" t="n">
         <f aca="false">IF(G20=0,0,K20-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E20&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>9.98930141843972</v>
+        <v>10.4964209452288</v>
       </c>
       <c r="O20" s="22" t="n">
         <f aca="false">G20*Paramètres!$C$25</f>
-        <v>18.9585957446809</v>
+        <v>17.4372371643136</v>
       </c>
       <c r="P20" s="6" t="str">
         <f aca="false">IF(G20=0,"Prix fournisseur manquant",IF(N20&lt;0,"Perte si vendu seul",IF(L20&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -5964,7 +5965,7 @@
       </c>
       <c r="G21" s="35" t="n">
         <f aca="false">'Tarifs Onsha-Sullab'!$O$24</f>
-        <v>2.6916524822695</v>
+        <v>2.47565712826675</v>
       </c>
       <c r="H21" s="22" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E21/(1+Paramètres!$C$6),E21)</f>
@@ -5980,23 +5981,23 @@
       </c>
       <c r="K21" s="17" t="n">
         <f aca="false">IF(G21=0,0,H21-G21-I21-J21)</f>
-        <v>7.04651418439717</v>
+        <v>7.26250953839992</v>
       </c>
       <c r="L21" s="36" t="n">
         <f aca="false">IF(H21=0,0,K21/H21)</f>
-        <v>0.710572858930807</v>
+        <v>0.732353903031925</v>
       </c>
       <c r="M21" s="33" t="n">
         <f aca="false">IF(G21=0,0,E21/G21)</f>
-        <v>4.42107592952206</v>
+        <v>4.80680457084597</v>
       </c>
       <c r="N21" s="17" t="n">
         <f aca="false">IF(G21=0,0,K21-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E21&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>2.16051418439717</v>
+        <v>2.37650953839992</v>
       </c>
       <c r="O21" s="22" t="n">
         <f aca="false">G21*Paramètres!$C$25</f>
-        <v>8.07495744680851</v>
+        <v>7.42697138480024</v>
       </c>
       <c r="P21" s="6" t="str">
         <f aca="false">IF(G21=0,"Prix fournisseur manquant",IF(N21&lt;0,"Perte si vendu seul",IF(L21&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
@@ -6318,7 +6319,7 @@
       </c>
       <c r="E6" s="35" t="n">
         <f aca="false">IF(B6="",0,C6*INDEX('Marges produits'!$G$5:$G$25,MATCH(B6,'Marges produits'!$B$5:$B$25,0)))</f>
-        <v>15.4477446808511</v>
+        <v>14.2081191709222</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6334,7 +6335,7 @@
       </c>
       <c r="E7" s="35" t="n">
         <f aca="false">IF(B7="",0,C7*INDEX('Marges produits'!$G$5:$G$25,MATCH(B7,'Marges produits'!$B$5:$B$25,0)))</f>
-        <v>11.0006666666667</v>
+        <v>10.1179030459597</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6423,7 +6424,7 @@
       </c>
       <c r="D16" s="22" t="n">
         <f aca="false">-SUM(E6:E11)</f>
-        <v>-26.4484113475177</v>
+        <v>-24.3260222168819</v>
       </c>
       <c r="F16" s="32"/>
     </row>
@@ -6479,7 +6480,7 @@
       </c>
       <c r="D22" s="17" t="n">
         <f aca="false">SUM(D15:D21)</f>
-        <v>30.6134219858156</v>
+        <v>32.7358111164514</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6488,7 +6489,7 @@
       </c>
       <c r="D23" s="36" t="n">
         <f aca="false">IF(D15=0,0,D22/D15)</f>
-        <v>0.455782957605195</v>
+        <v>0.487381803222601</v>
       </c>
     </row>
   </sheetData>
@@ -6652,7 +6653,7 @@
       </c>
       <c r="C17" s="35" t="n">
         <f aca="false">'Simulateur commande'!D22</f>
-        <v>30.6134219858156</v>
+        <v>32.7358111164514</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>343</v>

</xml_diff>

<commit_message>
Gestion : livraison Mondial Relay 5,90 €, transporteur 4 €, emballage 1 €, cadeau 1 €
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6qThdJp8fvnL986bvjdNe
</commit_message>
<xml_diff>
--- a/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
+++ b/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
@@ -169,7 +169,7 @@
     <t xml:space="preserve">Livraison payée par la cliente (TTC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Repris de tes tarifs Shopify : Mondial Relay 4,90 € (&lt; 500 g) ou 5,90 € (500 g à 1 kg), Colissimo 7,90 € ou 9,90 €. 4,90 € = le cas le plus courant.</t>
+    <t xml:space="preserve">Repris de tes tarifs Shopify : Mondial Relay 5,90 € (&lt; 1 kg, depuis le 14/10/2026), Colissimo 7,90 € ou 9,90 €. 5,90 € = le cas le plus courant.</t>
   </si>
   <si>
     <t xml:space="preserve">Livraison offerte à partir de (TTC)</t>
@@ -211,7 +211,7 @@
     <t xml:space="preserve">→ Emballage par colis (TTC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Calcul automatique.</t>
+    <t xml:space="preserve">Ton estimation réelle (14/10/2026). Le détail ci-dessus sert de repère.</t>
   </si>
   <si>
     <t xml:space="preserve">Petit cadeau / échantillon par colis (TTC)</t>
@@ -1426,10 +1426,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1479,6 +1475,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="174" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1939,53 +1939,53 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="19" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="26" t="s">
         <v>348</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>349</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>350</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="26" t="s">
         <v>351</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="26" t="s">
         <v>352</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="26" t="s">
         <v>353</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="26" t="s">
         <v>354</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="26" t="s">
         <v>355</v>
       </c>
-      <c r="I4" s="27" t="s">
+      <c r="I4" s="26" t="s">
         <v>238</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="26" t="s">
         <v>356</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="K4" s="26" t="s">
         <v>357</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="L4" s="26" t="s">
         <v>358</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="M4" s="26" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>360</v>
       </c>
       <c r="B5" s="8" t="s">
@@ -2009,11 +2009,11 @@
         <f aca="false">2*'Marges produits'!$G$11</f>
         <v>10.1179030459597</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E5/(1+Paramètres!$C$6),E5)</f>
         <v>19.9166666666667</v>
       </c>
-      <c r="I5" s="17" t="n">
+      <c r="I5" s="30" t="n">
         <f aca="false">H5-G5-E5*Paramètres!$C$11-H5*Paramètres!$C$13</f>
         <v>9.44026362070692</v>
       </c>
@@ -2021,13 +2021,13 @@
         <f aca="false">IF(H5=0,0,I5/H5)</f>
         <v>0.473988131583611</v>
       </c>
-      <c r="K5" s="17" t="n">
+      <c r="K5" s="30" t="n">
         <f aca="false">I5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>4.55426362070692</v>
+        <v>9.01843028737359</v>
       </c>
       <c r="L5" s="35" t="n">
         <f aca="false">'Marges produits'!$N$11</f>
-        <v>0.611548477020127</v>
+        <v>5.07571514368679</v>
       </c>
       <c r="M5" s="6" t="str">
         <f aca="false">IF(E5&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2035,7 +2035,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>363</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -2059,11 +2059,11 @@
         <f aca="false">4*'Marges produits'!$G$11</f>
         <v>20.2358060919195</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E6/(1+Paramètres!$C$6),E6)</f>
         <v>37.4166666666667</v>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="I6" s="30" t="n">
         <f aca="false">H6-G6-E6*Paramètres!$C$11-H6*Paramètres!$C$13</f>
         <v>16.5073605747472</v>
       </c>
@@ -2071,13 +2071,13 @@
         <f aca="false">IF(H6=0,0,I6/H6)</f>
         <v>0.441176674603488</v>
       </c>
-      <c r="K6" s="17" t="n">
+      <c r="K6" s="30" t="n">
         <f aca="false">I6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>11.6213605747472</v>
+        <v>16.0855272414138</v>
       </c>
       <c r="L6" s="35" t="n">
         <f aca="false">'Marges produits'!$N$11</f>
-        <v>0.611548477020127</v>
+        <v>5.07571514368679</v>
       </c>
       <c r="M6" s="6" t="str">
         <f aca="false">IF(E6&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2085,7 +2085,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>366</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -2109,11 +2109,11 @@
         <f aca="false">3*'Marges produits'!$G$13</f>
         <v>7.42697138480024</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E7/(1+Paramètres!$C$6),E7)</f>
         <v>14.9166666666667</v>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="I7" s="30" t="n">
         <f aca="false">H7-G7-E7*Paramètres!$C$11-H7*Paramètres!$C$13</f>
         <v>7.22119528186643</v>
       </c>
@@ -2121,13 +2121,13 @@
         <f aca="false">IF(H7=0,0,I7/H7)</f>
         <v>0.484102476996632</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="K7" s="30" t="n">
         <f aca="false">I7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>2.33519528186643</v>
+        <v>6.7993619485331</v>
       </c>
       <c r="L7" s="35" t="n">
         <f aca="false">'Marges produits'!$N$13</f>
-        <v>-1.71515712826675</v>
+        <v>2.74900953839992</v>
       </c>
       <c r="M7" s="6" t="str">
         <f aca="false">IF(E7&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2135,7 +2135,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="24" t="s">
         <v>369</v>
       </c>
       <c r="B8" s="8" t="s">
@@ -2159,11 +2159,11 @@
         <f aca="false">6*'Marges produits'!$G$13</f>
         <v>14.8539427696005</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E8/(1+Paramètres!$C$6),E8)</f>
         <v>29.0833333333333</v>
       </c>
-      <c r="I8" s="17" t="n">
+      <c r="I8" s="30" t="n">
         <f aca="false">H8-G8-E8*Paramètres!$C$11-H8*Paramètres!$C$13</f>
         <v>13.7058905637329</v>
       </c>
@@ -2171,13 +2171,13 @@
         <f aca="false">IF(H8=0,0,I8/H8)</f>
         <v>0.471262712793107</v>
       </c>
-      <c r="K8" s="17" t="n">
+      <c r="K8" s="30" t="n">
         <f aca="false">I8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>8.81989056373286</v>
+        <v>13.2840572303995</v>
       </c>
       <c r="L8" s="35" t="n">
         <f aca="false">'Marges produits'!$N$13</f>
-        <v>-1.71515712826675</v>
+        <v>2.74900953839992</v>
       </c>
       <c r="M8" s="6" t="str">
         <f aca="false">IF(E8&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2185,7 +2185,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="24" t="s">
         <v>372</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -2209,11 +2209,11 @@
         <f aca="false">1*'Marges produits'!$G$6+1*'Marges produits'!$G$8</f>
         <v>10.9790011775308</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E9/(1+Paramètres!$C$6),E9)</f>
         <v>24.9166666666667</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="30" t="n">
         <f aca="false">H9-G9-E9*Paramètres!$C$11-H9*Paramètres!$C$13</f>
         <v>13.4891654891359</v>
       </c>
@@ -2221,13 +2221,13 @@
         <f aca="false">IF(H9=0,0,I9/H9)</f>
         <v>0.541371190199433</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="30" t="n">
         <f aca="false">I9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>8.60316548913588</v>
+        <v>13.0673321558025</v>
       </c>
       <c r="L9" s="35" t="n">
         <f aca="false">'Marges produits'!$N$8</f>
-        <v>-0.767078858516071</v>
+        <v>3.6970878081506</v>
       </c>
       <c r="M9" s="6" t="str">
         <f aca="false">IF(E9&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2235,7 +2235,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="24" t="s">
         <v>375</v>
       </c>
       <c r="B10" s="8" t="s">
@@ -2259,11 +2259,11 @@
         <f aca="false">2*'Marges produits'!$G$7</f>
         <v>9.04153038149594</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E10/(1+Paramètres!$C$6),E10)</f>
         <v>20.75</v>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="I10" s="30" t="n">
         <f aca="false">H10-G10-E10*Paramètres!$C$11-H10*Paramètres!$C$13</f>
         <v>11.3349696185041</v>
       </c>
@@ -2271,13 +2271,13 @@
         <f aca="false">IF(H10=0,0,I10/H10)</f>
         <v>0.546263596072485</v>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="K10" s="30" t="n">
         <f aca="false">I10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>6.44896961850406</v>
+        <v>10.9131362851707</v>
       </c>
       <c r="L10" s="35" t="n">
         <f aca="false">'Marges produits'!$N$7</f>
-        <v>1.96806814258536</v>
+        <v>6.43223480925203</v>
       </c>
       <c r="M10" s="6" t="str">
         <f aca="false">IF(E10&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2285,7 +2285,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>378</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -2309,11 +2309,11 @@
         <f aca="false">1*'Marges produits'!$G$16+2*'Marges produits'!$G$11</f>
         <v>31.6453563352358</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H11" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E11/(1+Paramètres!$C$6),E11)</f>
         <v>62.4166666666667</v>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="I11" s="30" t="n">
         <f aca="false">H11-G11-E11*Paramètres!$C$11-H11*Paramètres!$C$13</f>
         <v>29.6478103314309</v>
       </c>
@@ -2321,13 +2321,13 @@
         <f aca="false">IF(H11=0,0,I11/H11)</f>
         <v>0.474998296364714</v>
       </c>
-      <c r="K11" s="17" t="n">
+      <c r="K11" s="30" t="n">
         <f aca="false">I11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>24.7618103314309</v>
+        <v>29.2259769980975</v>
       </c>
       <c r="L11" s="35" t="n">
         <f aca="false">'Marges produits'!$N$16</f>
-        <v>22.6047133773906</v>
+        <v>27.0688800440573</v>
       </c>
       <c r="M11" s="6" t="str">
         <f aca="false">IF(E11&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2335,7 +2335,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="24" t="s">
         <v>381</v>
       </c>
       <c r="B12" s="8" t="s">
@@ -2359,11 +2359,11 @@
         <f aca="false">1*'Marges produits'!$G$17+3*'Marges produits'!$G$13</f>
         <v>18.405972562331</v>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="H12" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E12/(1+Paramètres!$C$6),E12)</f>
         <v>37.4166666666667</v>
       </c>
-      <c r="I12" s="17" t="n">
+      <c r="I12" s="30" t="n">
         <f aca="false">H12-G12-E12*Paramètres!$C$11-H12*Paramètres!$C$13</f>
         <v>18.3371941043356</v>
       </c>
@@ -2371,13 +2371,13 @@
         <f aca="false">IF(H12=0,0,I12/H12)</f>
         <v>0.490080911474449</v>
       </c>
-      <c r="K12" s="17" t="n">
+      <c r="K12" s="30" t="n">
         <f aca="false">I12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>13.4511941043356</v>
+        <v>17.9153607710023</v>
       </c>
       <c r="L12" s="35" t="n">
         <f aca="false">'Marges produits'!$N$17</f>
-        <v>8.60316548913588</v>
+        <v>13.0673321558026</v>
       </c>
       <c r="M12" s="6" t="str">
         <f aca="false">IF(E12&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2590,7 +2590,7 @@
         <v>43</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>44</v>
@@ -2601,7 +2601,7 @@
         <v>45</v>
       </c>
       <c r="C15" s="14" t="n">
-        <v>4.9</v>
+        <v>5.9</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>46</v>
@@ -2677,9 +2677,8 @@
       <c r="B22" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="17" t="n">
-        <f aca="false">$C$17/$C$18+$C$19/$C$20+$C$21</f>
-        <v>1.875</v>
+      <c r="C22" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>60</v>
@@ -2690,7 +2689,7 @@
         <v>61</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>62</v>
@@ -2711,7 +2710,7 @@
       <c r="B25" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C25" s="17" t="n">
         <v>3</v>
       </c>
       <c r="D25" s="8" t="s">
@@ -2730,7 +2729,7 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="18" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2775,7 +2774,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2851,15 +2850,15 @@
       <c r="B9" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="20" t="n">
         <f aca="false">IF(C7="USD",Paramètres!$C$7,IF(C7="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="20" t="n">
         <f aca="false">IF(D7="USD",Paramètres!$C$7,IF(D7="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="20" t="n">
         <f aca="false">IF(E7="USD",Paramètres!$C$7,IF(E7="KRW",Paramètres!$C$8,1))</f>
         <v>1</v>
       </c>
@@ -2871,15 +2870,15 @@
       <c r="B10" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="21" t="n">
         <f aca="false">C6*C9</f>
         <v>2862.94</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="21" t="n">
         <f aca="false">D6*D9</f>
         <v>1965.1</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="21" t="n">
         <f aca="false">E6*E9</f>
         <v>435</v>
       </c>
@@ -2889,7 +2888,7 @@
       <c r="B11" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="21" t="n">
         <f aca="false">773.61*Paramètres!$C$7</f>
         <v>665.3046</v>
       </c>
@@ -2958,15 +2957,15 @@
       <c r="B15" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">IF(C8="UE",0,Paramètres!$C$10)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="22" t="n">
         <f aca="false">IF(D8="UE",0,Paramètres!$C$10)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="22" t="n">
         <f aca="false">IF(E8="UE",0,Paramètres!$C$10)</f>
         <v>0</v>
       </c>
@@ -2978,15 +2977,15 @@
       <c r="B16" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="21" t="n">
         <f aca="false">(C10+C11+C12)*C15</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="D16" s="21" t="n">
         <f aca="false">(D10+D11+D12)*D15</f>
         <v>0</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="21" t="n">
         <f aca="false">(E10+E11+E12)*E15</f>
         <v>0</v>
       </c>
@@ -2998,15 +2997,15 @@
       <c r="B17" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="21" t="n">
         <f aca="false">IF(C8="UE",0,(C10+C11+C12+C16)*Paramètres!$C$6)</f>
         <v>705.64892</v>
       </c>
-      <c r="D17" s="22" t="n">
+      <c r="D17" s="21" t="n">
         <f aca="false">IF(D8="UE",0,(D10+D11+D12+D16)*Paramètres!$C$6)</f>
         <v>443.02</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="21" t="n">
         <f aca="false">IF(E8="UE",0,(E10+E11+E12+E16)*Paramètres!$C$6)</f>
         <v>91.1</v>
       </c>
@@ -3018,15 +3017,15 @@
       <c r="B18" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="21" t="n">
         <f aca="false">SUM(C10:C14)+C16+C17</f>
         <v>4288.89352</v>
       </c>
-      <c r="D18" s="22" t="n">
+      <c r="D18" s="21" t="n">
         <f aca="false">SUM(D10:D14)+D16+D17</f>
         <v>2713.12</v>
       </c>
-      <c r="E18" s="22" t="n">
+      <c r="E18" s="21" t="n">
         <f aca="false">SUM(E10:E14)+E16+E17</f>
         <v>586.6</v>
       </c>
@@ -3036,15 +3035,15 @@
       <c r="B19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="23" t="n">
         <f aca="false">IF(C10=0,1,(C18-C17)/C10)</f>
         <v>1.25159612146954</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="23" t="n">
         <f aca="false">IF(D10=0,1,(D18-D17)/D10)</f>
         <v>1.15520838634166</v>
       </c>
-      <c r="E19" s="24" t="n">
+      <c r="E19" s="23" t="n">
         <f aca="false">IF(E10=0,1,(E18-E17)/E10)</f>
         <v>1.13908045977012</v>
       </c>
@@ -3056,15 +3055,15 @@
       <c r="B20" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="23" t="n">
         <f aca="false">IF(C10=0,1,C18/C10)</f>
         <v>1.4980731415957</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="23" t="n">
         <f aca="false">IF(D10=0,1,D18/D10)</f>
         <v>1.38065238410259</v>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="E20" s="23" t="n">
         <f aca="false">IF(E10=0,1,E18/E10)</f>
         <v>1.34850574712644</v>
       </c>
@@ -3073,18 +3072,18 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="26" t="n">
+      <c r="C21" s="25" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),C19,C20)</f>
         <v>1.25159612146954</v>
       </c>
-      <c r="D21" s="26" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),D19,D20)</f>
         <v>1.15520838634166</v>
       </c>
-      <c r="E21" s="26" t="n">
+      <c r="E21" s="25" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E19,E20)</f>
         <v>1.13908045977012</v>
       </c>
@@ -3143,54 +3142,54 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="19" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="26" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="I4" s="27" t="s">
+      <c r="I4" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="K4" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="L4" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="M4" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="N4" s="27" t="s">
+      <c r="N4" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="O4" s="27" t="s">
+      <c r="O4" s="26" t="s">
         <v>126</v>
       </c>
     </row>
@@ -3204,42 +3203,42 @@
       <c r="C5" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="27" t="n">
         <v>6.5</v>
       </c>
-      <c r="E5" s="29" t="n">
+      <c r="E5" s="28" t="n">
         <f aca="false">D5*F5</f>
         <v>260</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G5" s="27" t="n">
         <v>5.5</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I5" s="29" t="n">
+      <c r="I5" s="28" t="n">
         <f aca="false">G5*H5</f>
         <v>5500</v>
       </c>
-      <c r="J5" s="28" t="n">
+      <c r="J5" s="27" t="n">
         <v>15.5</v>
       </c>
-      <c r="K5" s="30" t="n">
+      <c r="K5" s="29" t="n">
         <v>7.5</v>
       </c>
       <c r="L5" s="6"/>
-      <c r="M5" s="29" t="n">
+      <c r="M5" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G5,D5)</f>
         <v>6.5</v>
       </c>
-      <c r="N5" s="22" t="n">
+      <c r="N5" s="21" t="n">
         <f aca="false">M5*Paramètres!$C$7</f>
         <v>5.59</v>
       </c>
-      <c r="O5" s="17" t="n">
+      <c r="O5" s="30" t="n">
         <f aca="false">N5*Import!$C$21</f>
         <v>6.99642231901472</v>
       </c>
@@ -3254,42 +3253,42 @@
       <c r="C6" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="27" t="n">
         <v>3.7</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="28" t="n">
         <f aca="false">D6*F6</f>
         <v>185</v>
       </c>
       <c r="F6" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="27" t="n">
         <v>3.2</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I6" s="29" t="n">
+      <c r="I6" s="28" t="n">
         <f aca="false">G6*H6</f>
         <v>3200</v>
       </c>
-      <c r="J6" s="28" t="n">
+      <c r="J6" s="27" t="n">
         <v>6.54</v>
       </c>
-      <c r="K6" s="30" t="n">
+      <c r="K6" s="29" t="n">
         <v>5.5</v>
       </c>
       <c r="L6" s="6"/>
-      <c r="M6" s="29" t="n">
+      <c r="M6" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G6,D6)</f>
         <v>3.7</v>
       </c>
-      <c r="N6" s="22" t="n">
+      <c r="N6" s="21" t="n">
         <f aca="false">M6*Paramètres!$C$7</f>
         <v>3.182</v>
       </c>
-      <c r="O6" s="17" t="n">
+      <c r="O6" s="30" t="n">
         <f aca="false">N6*Import!$C$21</f>
         <v>3.98257885851607</v>
       </c>
@@ -3304,44 +3303,44 @@
       <c r="C7" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="27" t="n">
         <v>4.2</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="28" t="n">
         <f aca="false">D7*F7</f>
         <v>226.8</v>
       </c>
       <c r="F7" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G7" s="27" t="n">
         <v>3.8</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>1026</v>
       </c>
-      <c r="I7" s="29" t="n">
+      <c r="I7" s="28" t="n">
         <f aca="false">G7*H7</f>
         <v>3898.8</v>
       </c>
-      <c r="J7" s="28" t="n">
+      <c r="J7" s="27" t="n">
         <v>9.5</v>
       </c>
-      <c r="K7" s="30" t="n">
+      <c r="K7" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="M7" s="29" t="n">
+      <c r="M7" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G7,D7)</f>
         <v>4.2</v>
       </c>
-      <c r="N7" s="22" t="n">
+      <c r="N7" s="21" t="n">
         <f aca="false">M7*Paramètres!$C$7</f>
         <v>3.612</v>
       </c>
-      <c r="O7" s="17" t="n">
+      <c r="O7" s="30" t="n">
         <f aca="false">N7*Import!$C$21</f>
         <v>4.52076519074797</v>
       </c>
@@ -3356,44 +3355,44 @@
       <c r="C8" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="28" t="n">
         <f aca="false">D8*F8</f>
         <v>144</v>
       </c>
       <c r="F8" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="27" t="n">
         <v>5</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I8" s="29" t="n">
+      <c r="I8" s="28" t="n">
         <f aca="false">G8*H8</f>
         <v>5040</v>
       </c>
-      <c r="J8" s="28" t="n">
+      <c r="J8" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="K8" s="30" t="n">
+      <c r="K8" s="29" t="n">
         <v>8</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="M8" s="29" t="n">
+      <c r="M8" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G8,D8)</f>
         <v>6</v>
       </c>
-      <c r="N8" s="22" t="n">
+      <c r="N8" s="21" t="n">
         <f aca="false">M8*Paramètres!$C$7</f>
         <v>5.16</v>
       </c>
-      <c r="O8" s="17" t="n">
+      <c r="O8" s="30" t="n">
         <f aca="false">N8*Import!$C$21</f>
         <v>6.45823598678282</v>
       </c>
@@ -3408,44 +3407,44 @@
       <c r="C9" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="27" t="n">
         <v>6.5</v>
       </c>
-      <c r="E9" s="29" t="n">
+      <c r="E9" s="28" t="n">
         <f aca="false">D9*F9</f>
         <v>156</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G9" s="27" t="n">
         <v>5.2</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I9" s="29" t="n">
+      <c r="I9" s="28" t="n">
         <f aca="false">G9*H9</f>
         <v>5241.6</v>
       </c>
-      <c r="J9" s="28" t="n">
+      <c r="J9" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="K9" s="30" t="n">
+      <c r="K9" s="29" t="n">
         <v>9</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="M9" s="29" t="n">
+      <c r="M9" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G9,D9)</f>
         <v>6.5</v>
       </c>
-      <c r="N9" s="22" t="n">
+      <c r="N9" s="21" t="n">
         <f aca="false">M9*Paramètres!$C$7</f>
         <v>5.59</v>
       </c>
-      <c r="O9" s="17" t="n">
+      <c r="O9" s="30" t="n">
         <f aca="false">N9*Import!$C$21</f>
         <v>6.99642231901472</v>
       </c>
@@ -3460,42 +3459,42 @@
       <c r="C10" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="27" t="n">
         <v>10.2</v>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="28" t="n">
         <f aca="false">D10*F10</f>
         <v>183.6</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="27" t="n">
         <v>9.2</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I10" s="29" t="n">
+      <c r="I10" s="28" t="n">
         <f aca="false">G10*H10</f>
         <v>9273.6</v>
       </c>
-      <c r="J10" s="28" t="n">
+      <c r="J10" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="K10" s="30" t="n">
+      <c r="K10" s="29" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="6"/>
-      <c r="M10" s="29" t="n">
+      <c r="M10" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G10,D10)</f>
         <v>10.2</v>
       </c>
-      <c r="N10" s="22" t="n">
+      <c r="N10" s="21" t="n">
         <f aca="false">M10*Paramètres!$C$7</f>
         <v>8.772</v>
       </c>
-      <c r="O10" s="17" t="n">
+      <c r="O10" s="30" t="n">
         <f aca="false">N10*Import!$C$21</f>
         <v>10.9790011775308</v>
       </c>
@@ -3510,42 +3509,42 @@
       <c r="C11" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="28" t="n">
+      <c r="D11" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="28" t="n">
         <f aca="false">D11*F11</f>
         <v>460</v>
       </c>
       <c r="F11" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="G11" s="28" t="n">
+      <c r="G11" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I11" s="29" t="n">
+      <c r="I11" s="28" t="n">
         <f aca="false">G11*H11</f>
         <v>1800</v>
       </c>
-      <c r="J11" s="28" t="n">
+      <c r="J11" s="27" t="n">
         <v>6.54</v>
       </c>
-      <c r="K11" s="30" t="n">
+      <c r="K11" s="29" t="n">
         <v>5.5</v>
       </c>
       <c r="L11" s="6"/>
-      <c r="M11" s="29" t="n">
+      <c r="M11" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G11,D11)</f>
         <v>2.3</v>
       </c>
-      <c r="N11" s="22" t="n">
+      <c r="N11" s="21" t="n">
         <f aca="false">M11*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O11" s="17" t="n">
+      <c r="O11" s="30" t="n">
         <f aca="false">N11*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -3560,42 +3559,42 @@
       <c r="C12" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="28" t="n">
         <f aca="false">D12*F12</f>
         <v>460</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I12" s="29" t="n">
+      <c r="I12" s="28" t="n">
         <f aca="false">G12*H12</f>
         <v>1800</v>
       </c>
-      <c r="J12" s="28" t="n">
+      <c r="J12" s="27" t="n">
         <v>6.54</v>
       </c>
-      <c r="K12" s="30" t="n">
+      <c r="K12" s="29" t="n">
         <v>5.5</v>
       </c>
       <c r="L12" s="6"/>
-      <c r="M12" s="29" t="n">
+      <c r="M12" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G12,D12)</f>
         <v>2.3</v>
       </c>
-      <c r="N12" s="22" t="n">
+      <c r="N12" s="21" t="n">
         <f aca="false">M12*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O12" s="17" t="n">
+      <c r="O12" s="30" t="n">
         <f aca="false">N12*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -3610,42 +3609,42 @@
       <c r="C13" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="D13" s="28" t="n">
+      <c r="D13" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E13" s="29" t="n">
+      <c r="E13" s="28" t="n">
         <f aca="false">D13*F13</f>
         <v>460</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="G13" s="28" t="n">
+      <c r="G13" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I13" s="29" t="n">
+      <c r="I13" s="28" t="n">
         <f aca="false">G13*H13</f>
         <v>1800</v>
       </c>
-      <c r="J13" s="28" t="n">
+      <c r="J13" s="27" t="n">
         <v>6.54</v>
       </c>
-      <c r="K13" s="30" t="n">
+      <c r="K13" s="29" t="n">
         <v>5.5</v>
       </c>
       <c r="L13" s="6"/>
-      <c r="M13" s="29" t="n">
+      <c r="M13" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G13,D13)</f>
         <v>2.3</v>
       </c>
-      <c r="N13" s="22" t="n">
+      <c r="N13" s="21" t="n">
         <f aca="false">M13*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O13" s="17" t="n">
+      <c r="O13" s="30" t="n">
         <f aca="false">N13*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -3660,42 +3659,42 @@
       <c r="C14" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D14" s="28" t="n">
+      <c r="D14" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E14" s="29" t="n">
+      <c r="E14" s="28" t="n">
         <f aca="false">D14*F14</f>
         <v>460</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="G14" s="28" t="n">
+      <c r="G14" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I14" s="29" t="n">
+      <c r="I14" s="28" t="n">
         <f aca="false">G14*H14</f>
         <v>1800</v>
       </c>
-      <c r="J14" s="28" t="n">
+      <c r="J14" s="27" t="n">
         <v>6.54</v>
       </c>
-      <c r="K14" s="30" t="n">
+      <c r="K14" s="29" t="n">
         <v>5.5</v>
       </c>
       <c r="L14" s="6"/>
-      <c r="M14" s="29" t="n">
+      <c r="M14" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G14,D14)</f>
         <v>2.3</v>
       </c>
-      <c r="N14" s="22" t="n">
+      <c r="N14" s="21" t="n">
         <f aca="false">M14*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O14" s="17" t="n">
+      <c r="O14" s="30" t="n">
         <f aca="false">N14*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -3710,42 +3709,42 @@
       <c r="C15" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="D15" s="28" t="n">
+      <c r="D15" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E15" s="29" t="n">
+      <c r="E15" s="28" t="n">
         <f aca="false">D15*F15</f>
         <v>460</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="G15" s="28" t="n">
+      <c r="G15" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="I15" s="29" t="n">
+      <c r="I15" s="28" t="n">
         <f aca="false">G15*H15</f>
         <v>1800</v>
       </c>
-      <c r="J15" s="28" t="n">
+      <c r="J15" s="27" t="n">
         <v>6.15</v>
       </c>
-      <c r="K15" s="30" t="n">
+      <c r="K15" s="29" t="n">
         <v>10.5</v>
       </c>
       <c r="L15" s="6"/>
-      <c r="M15" s="29" t="n">
+      <c r="M15" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G15,D15)</f>
         <v>2.3</v>
       </c>
-      <c r="N15" s="22" t="n">
+      <c r="N15" s="21" t="n">
         <f aca="false">M15*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O15" s="17" t="n">
+      <c r="O15" s="30" t="n">
         <f aca="false">N15*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -3760,42 +3759,42 @@
       <c r="C16" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="D16" s="28" t="n">
+      <c r="D16" s="27" t="n">
         <v>6.2</v>
       </c>
-      <c r="E16" s="29" t="n">
+      <c r="E16" s="28" t="n">
         <f aca="false">D16*F16</f>
         <v>260.4</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="G16" s="28" t="n">
+      <c r="G16" s="27" t="n">
         <v>5.2</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I16" s="29" t="n">
+      <c r="I16" s="28" t="n">
         <f aca="false">G16*H16</f>
         <v>5241.6</v>
       </c>
-      <c r="J16" s="28" t="n">
+      <c r="J16" s="27" t="n">
         <v>12.5</v>
       </c>
-      <c r="K16" s="30" t="n">
+      <c r="K16" s="29" t="n">
         <v>8.5</v>
       </c>
       <c r="L16" s="6"/>
-      <c r="M16" s="29" t="n">
+      <c r="M16" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G16,D16)</f>
         <v>6.2</v>
       </c>
-      <c r="N16" s="22" t="n">
+      <c r="N16" s="21" t="n">
         <f aca="false">M16*Paramètres!$C$7</f>
         <v>5.332</v>
       </c>
-      <c r="O16" s="17" t="n">
+      <c r="O16" s="30" t="n">
         <f aca="false">N16*Import!$C$21</f>
         <v>6.67351051967558</v>
       </c>
@@ -3810,42 +3809,42 @@
       <c r="C17" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="D17" s="28" t="n">
+      <c r="D17" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E17" s="29" t="n">
+      <c r="E17" s="28" t="n">
         <f aca="false">D17*F17</f>
         <v>240</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="G17" s="28" t="n">
+      <c r="G17" s="27" t="n">
         <v>18.5</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="I17" s="28" t="n">
         <f aca="false">G17*H17</f>
         <v>18648</v>
       </c>
-      <c r="J17" s="28" t="n">
+      <c r="J17" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="K17" s="30" t="n">
+      <c r="K17" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="L17" s="6"/>
-      <c r="M17" s="29" t="n">
+      <c r="M17" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G17,D17)</f>
         <v>20</v>
       </c>
-      <c r="N17" s="22" t="n">
+      <c r="N17" s="21" t="n">
         <f aca="false">M17*Paramètres!$C$7</f>
         <v>17.2</v>
       </c>
-      <c r="O17" s="17" t="n">
+      <c r="O17" s="30" t="n">
         <f aca="false">N17*Import!$C$21</f>
         <v>21.5274532892761</v>
       </c>
@@ -3860,42 +3859,42 @@
       <c r="C18" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D18" s="28" t="n">
+      <c r="D18" s="27" t="n">
         <v>4.7</v>
       </c>
-      <c r="E18" s="29" t="n">
+      <c r="E18" s="28" t="n">
         <f aca="false">D18*F18</f>
         <v>338.4</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="G18" s="28" t="n">
+      <c r="G18" s="27" t="n">
         <v>4.2</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I18" s="29" t="n">
+      <c r="I18" s="28" t="n">
         <f aca="false">G18*H18</f>
         <v>4233.6</v>
       </c>
-      <c r="J18" s="28" t="n">
+      <c r="J18" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="K18" s="30" t="n">
+      <c r="K18" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="L18" s="6"/>
-      <c r="M18" s="29" t="n">
+      <c r="M18" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G18,D18)</f>
         <v>4.7</v>
       </c>
-      <c r="N18" s="22" t="n">
+      <c r="N18" s="21" t="n">
         <f aca="false">M18*Paramètres!$C$7</f>
         <v>4.042</v>
       </c>
-      <c r="O18" s="17" t="n">
+      <c r="O18" s="30" t="n">
         <f aca="false">N18*Import!$C$21</f>
         <v>5.05895152297987</v>
       </c>
@@ -3910,42 +3909,42 @@
       <c r="C19" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D19" s="28" t="n">
+      <c r="D19" s="27" t="n">
         <v>4.7</v>
       </c>
-      <c r="E19" s="29" t="n">
+      <c r="E19" s="28" t="n">
         <f aca="false">D19*F19</f>
         <v>338.4</v>
       </c>
       <c r="F19" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="G19" s="28" t="n">
+      <c r="G19" s="27" t="n">
         <v>4.2</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I19" s="29" t="n">
+      <c r="I19" s="28" t="n">
         <f aca="false">G19*H19</f>
         <v>4233.6</v>
       </c>
-      <c r="J19" s="28" t="n">
+      <c r="J19" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="K19" s="30" t="n">
+      <c r="K19" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="L19" s="6"/>
-      <c r="M19" s="29" t="n">
+      <c r="M19" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G19,D19)</f>
         <v>4.7</v>
       </c>
-      <c r="N19" s="22" t="n">
+      <c r="N19" s="21" t="n">
         <f aca="false">M19*Paramètres!$C$7</f>
         <v>4.042</v>
       </c>
-      <c r="O19" s="17" t="n">
+      <c r="O19" s="30" t="n">
         <f aca="false">N19*Import!$C$21</f>
         <v>5.05895152297987</v>
       </c>
@@ -3960,42 +3959,42 @@
       <c r="C20" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="D20" s="28" t="n">
+      <c r="D20" s="27" t="n">
         <v>4.7</v>
       </c>
-      <c r="E20" s="29" t="n">
+      <c r="E20" s="28" t="n">
         <f aca="false">D20*F20</f>
         <v>338.4</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="G20" s="27" t="n">
         <v>4.2</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I20" s="29" t="n">
+      <c r="I20" s="28" t="n">
         <f aca="false">G20*H20</f>
         <v>4233.6</v>
       </c>
-      <c r="J20" s="28" t="n">
+      <c r="J20" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="K20" s="30" t="n">
+      <c r="K20" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="L20" s="6"/>
-      <c r="M20" s="29" t="n">
+      <c r="M20" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G20,D20)</f>
         <v>4.7</v>
       </c>
-      <c r="N20" s="22" t="n">
+      <c r="N20" s="21" t="n">
         <f aca="false">M20*Paramètres!$C$7</f>
         <v>4.042</v>
       </c>
-      <c r="O20" s="17" t="n">
+      <c r="O20" s="30" t="n">
         <f aca="false">N20*Import!$C$21</f>
         <v>5.05895152297987</v>
       </c>
@@ -4010,42 +4009,42 @@
       <c r="C21" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D21" s="28" t="n">
+      <c r="D21" s="27" t="n">
         <v>4.7</v>
       </c>
-      <c r="E21" s="29" t="n">
+      <c r="E21" s="28" t="n">
         <f aca="false">D21*F21</f>
         <v>338.4</v>
       </c>
       <c r="F21" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="G21" s="28" t="n">
+      <c r="G21" s="27" t="n">
         <v>4.2</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I21" s="29" t="n">
+      <c r="I21" s="28" t="n">
         <f aca="false">G21*H21</f>
         <v>4233.6</v>
       </c>
-      <c r="J21" s="28" t="n">
+      <c r="J21" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="K21" s="30" t="n">
+      <c r="K21" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="L21" s="6"/>
-      <c r="M21" s="29" t="n">
+      <c r="M21" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G21,D21)</f>
         <v>4.7</v>
       </c>
-      <c r="N21" s="22" t="n">
+      <c r="N21" s="21" t="n">
         <f aca="false">M21*Paramètres!$C$7</f>
         <v>4.042</v>
       </c>
-      <c r="O21" s="17" t="n">
+      <c r="O21" s="30" t="n">
         <f aca="false">N21*Import!$C$21</f>
         <v>5.05895152297987</v>
       </c>
@@ -4060,42 +4059,42 @@
       <c r="C22" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="D22" s="28" t="n">
+      <c r="D22" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E22" s="29" t="n">
+      <c r="E22" s="28" t="n">
         <f aca="false">D22*F22</f>
         <v>165.6</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="G22" s="28" t="n">
+      <c r="G22" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I22" s="29" t="n">
+      <c r="I22" s="28" t="n">
         <f aca="false">G22*H22</f>
         <v>1814.4</v>
       </c>
-      <c r="J22" s="28" t="n">
+      <c r="J22" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="K22" s="30" t="n">
+      <c r="K22" s="29" t="n">
         <v>8.5</v>
       </c>
       <c r="L22" s="6"/>
-      <c r="M22" s="29" t="n">
+      <c r="M22" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G22,D22)</f>
         <v>2.3</v>
       </c>
-      <c r="N22" s="22" t="n">
+      <c r="N22" s="21" t="n">
         <f aca="false">M22*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O22" s="17" t="n">
+      <c r="O22" s="30" t="n">
         <f aca="false">N22*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -4110,44 +4109,44 @@
       <c r="C23" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D23" s="28" t="n">
+      <c r="D23" s="27" t="n">
         <v>5.4</v>
       </c>
-      <c r="E23" s="29" t="n">
+      <c r="E23" s="28" t="n">
         <f aca="false">D23*F23</f>
         <v>388.8</v>
       </c>
       <c r="F23" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="G23" s="28" t="n">
+      <c r="G23" s="27" t="n">
         <v>4.6</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>1008</v>
       </c>
-      <c r="I23" s="29" t="n">
+      <c r="I23" s="28" t="n">
         <f aca="false">G23*H23</f>
         <v>4636.8</v>
       </c>
-      <c r="J23" s="28" t="n">
+      <c r="J23" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="K23" s="30" t="n">
+      <c r="K23" s="29" t="n">
         <v>9</v>
       </c>
       <c r="L23" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="M23" s="29" t="n">
+      <c r="M23" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G23,D23)</f>
         <v>5.4</v>
       </c>
-      <c r="N23" s="22" t="n">
+      <c r="N23" s="21" t="n">
         <f aca="false">M23*Paramètres!$C$7</f>
         <v>4.644</v>
       </c>
-      <c r="O23" s="17" t="n">
+      <c r="O23" s="30" t="n">
         <f aca="false">N23*Import!$C$21</f>
         <v>5.81241238810454</v>
       </c>
@@ -4162,44 +4161,44 @@
       <c r="C24" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="D24" s="28" t="n">
+      <c r="D24" s="27" t="n">
         <v>2.3</v>
       </c>
-      <c r="E24" s="29" t="n">
+      <c r="E24" s="28" t="n">
         <f aca="false">D24*F24</f>
         <v>487.6</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>212</v>
       </c>
-      <c r="G24" s="28" t="n">
+      <c r="G24" s="27" t="n">
         <v>1.9</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>1060</v>
       </c>
-      <c r="I24" s="29" t="n">
+      <c r="I24" s="28" t="n">
         <f aca="false">G24*H24</f>
         <v>2014</v>
       </c>
-      <c r="J24" s="28" t="n">
+      <c r="J24" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="K24" s="30" t="n">
+      <c r="K24" s="29" t="n">
         <v>8.5</v>
       </c>
       <c r="L24" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="M24" s="29" t="n">
+      <c r="M24" s="28" t="n">
         <f aca="false">IF(Paramètres!$C$9="MOQ",G24,D24)</f>
         <v>2.3</v>
       </c>
-      <c r="N24" s="22" t="n">
+      <c r="N24" s="21" t="n">
         <f aca="false">M24*Paramètres!$C$7</f>
         <v>1.978</v>
       </c>
-      <c r="O24" s="17" t="n">
+      <c r="O24" s="30" t="n">
         <f aca="false">N24*Import!$C$21</f>
         <v>2.47565712826675</v>
       </c>
@@ -4242,45 +4241,45 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="19" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>172</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="26" t="s">
         <v>174</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="26" t="s">
         <v>176</v>
       </c>
-      <c r="I4" s="27" t="s">
+      <c r="I4" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="K4" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="L4" s="26" t="s">
         <v>126</v>
       </c>
     </row>
@@ -4312,15 +4311,15 @@
       <c r="I5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="20" t="n">
         <f aca="false">IF(E5="USD",Paramètres!$C$7,IF(E5="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="21" t="n">
         <f aca="false">D5*J5</f>
         <v>12.47</v>
       </c>
-      <c r="L5" s="17" t="n">
+      <c r="L5" s="30" t="n">
         <f aca="false">K5*Import!$D$21</f>
         <v>14.4054485776805</v>
       </c>
@@ -4353,15 +4352,15 @@
       <c r="I6" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="20" t="n">
         <f aca="false">IF(E6="USD",Paramètres!$C$7,IF(E6="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="K6" s="21" t="n">
         <f aca="false">D6*J6</f>
         <v>15.91</v>
       </c>
-      <c r="L6" s="17" t="n">
+      <c r="L6" s="30" t="n">
         <f aca="false">K6*Import!$D$21</f>
         <v>18.3793654266958</v>
       </c>
@@ -4394,15 +4393,15 @@
       <c r="I7" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="20" t="n">
         <f aca="false">IF(E7="USD",Paramètres!$C$7,IF(E7="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="K7" s="22" t="n">
+      <c r="K7" s="21" t="n">
         <f aca="false">D7*J7</f>
         <v>30.1</v>
       </c>
-      <c r="L7" s="17" t="n">
+      <c r="L7" s="30" t="n">
         <f aca="false">K7*Import!$D$21</f>
         <v>34.771772428884</v>
       </c>
@@ -4435,15 +4434,15 @@
       <c r="I8" s="15" t="n">
         <v>130</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="20" t="n">
         <f aca="false">IF(E8="USD",Paramètres!$C$7,IF(E8="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="K8" s="21" t="n">
         <f aca="false">D8*J8</f>
         <v>5.59</v>
       </c>
-      <c r="L8" s="17" t="n">
+      <c r="L8" s="30" t="n">
         <f aca="false">K8*Import!$D$21</f>
         <v>6.45761487964989</v>
       </c>
@@ -4476,15 +4475,15 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="J9" s="20" t="n">
         <f aca="false">IF(E9="USD",Paramètres!$C$7,IF(E9="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="K9" s="22" t="n">
+      <c r="K9" s="21" t="n">
         <f aca="false">D9*J9</f>
         <v>4.73</v>
       </c>
-      <c r="L9" s="17" t="n">
+      <c r="L9" s="30" t="n">
         <f aca="false">K9*Import!$D$21</f>
         <v>5.46413566739606</v>
       </c>
@@ -4517,15 +4516,15 @@
       <c r="I10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="20" t="n">
         <f aca="false">IF(E10="USD",Paramètres!$C$7,IF(E10="KRW",Paramètres!$C$8,1))</f>
         <v>0.86</v>
       </c>
-      <c r="K10" s="22" t="n">
+      <c r="K10" s="21" t="n">
         <f aca="false">D10*J10</f>
         <v>11.18</v>
       </c>
-      <c r="L10" s="17" t="n">
+      <c r="L10" s="30" t="n">
         <f aca="false">K10*Import!$D$21</f>
         <v>12.9152297592998</v>
       </c>
@@ -4623,33 +4622,33 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="19" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>209</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="26" t="s">
         <v>214</v>
       </c>
     </row>
@@ -4663,11 +4662,11 @@
       <c r="C5" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="21" t="n">
         <f aca="false">B5*C5</f>
         <v>105</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="30" t="n">
         <f aca="false">C5*Import!$E$21</f>
         <v>17.0862068965517</v>
       </c>
@@ -4688,11 +4687,11 @@
       <c r="C6" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="21" t="n">
         <f aca="false">B6*C6</f>
         <v>100</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="30" t="n">
         <f aca="false">C6*Import!$E$21</f>
         <v>11.3908045977012</v>
       </c>
@@ -4713,11 +4712,11 @@
       <c r="C7" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="21" t="n">
         <f aca="false">B7*C7</f>
         <v>50</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="30" t="n">
         <f aca="false">C7*Import!$E$21</f>
         <v>11.3908045977012</v>
       </c>
@@ -4738,11 +4737,11 @@
       <c r="C8" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="21" t="n">
         <f aca="false">B8*C8</f>
         <v>50</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="30" t="n">
         <f aca="false">C8*Import!$E$21</f>
         <v>11.3908045977012</v>
       </c>
@@ -4763,11 +4762,11 @@
       <c r="C9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="21" t="n">
         <f aca="false">B9*C9</f>
         <v>50</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="30" t="n">
         <f aca="false">C9*Import!$E$21</f>
         <v>5.69540229885058</v>
       </c>
@@ -4790,11 +4789,11 @@
       <c r="C10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="21" t="n">
         <f aca="false">B10*C10</f>
         <v>40</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="30" t="n">
         <f aca="false">C10*Import!$E$21</f>
         <v>4.55632183908046</v>
       </c>
@@ -4817,11 +4816,11 @@
       <c r="C11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D11" s="21" t="n">
         <f aca="false">B11*C11</f>
         <v>40</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="30" t="n">
         <f aca="false">C11*Import!$E$21</f>
         <v>4.55632183908046</v>
       </c>
@@ -4835,10 +4834,10 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="24" t="s">
         <v>223</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="30" t="n">
         <f aca="false">SUM(D5:D11)</f>
         <v>435</v>
       </c>
@@ -4852,10 +4851,10 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="30" t="n">
         <f aca="false">D12+D13</f>
         <v>455.5</v>
       </c>
@@ -4913,57 +4912,57 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="19" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="26" t="s">
         <v>229</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>230</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>231</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="26" t="s">
         <v>232</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="26" t="s">
         <v>233</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="26" t="s">
         <v>234</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="26" t="s">
         <v>235</v>
       </c>
-      <c r="I4" s="27" t="s">
+      <c r="I4" s="26" t="s">
         <v>236</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="26" t="s">
         <v>237</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="K4" s="26" t="s">
         <v>238</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="L4" s="26" t="s">
         <v>239</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="M4" s="26" t="s">
         <v>240</v>
       </c>
-      <c r="N4" s="27" t="s">
+      <c r="N4" s="26" t="s">
         <v>241</v>
       </c>
-      <c r="O4" s="27" t="s">
+      <c r="O4" s="26" t="s">
         <v>242</v>
       </c>
-      <c r="P4" s="27" t="s">
+      <c r="P4" s="26" t="s">
         <v>243</v>
       </c>
     </row>
@@ -4991,19 +4990,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$16</f>
         <v>6.67351051967558</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E5/(1+Paramètres!$C$6),E5)</f>
         <v>19.9166666666667</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <f aca="false">E5*Paramètres!$C$11</f>
         <v>0.3585</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="21" t="n">
         <f aca="false">H5*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K5" s="17" t="n">
+      <c r="K5" s="30" t="n">
         <f aca="false">IF(G5=0,0,H5-G5-I5-J5)</f>
         <v>12.8846561469911</v>
       </c>
@@ -5015,11 +5014,11 @@
         <f aca="false">IF(G5=0,0,E5/G5)</f>
         <v>3.58132349226624</v>
       </c>
-      <c r="N5" s="17" t="n">
+      <c r="N5" s="30" t="n">
         <f aca="false">IF(G5=0,0,K5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>7.99865614699109</v>
-      </c>
-      <c r="O5" s="22" t="n">
+        <v>12.4628228136578</v>
+      </c>
+      <c r="O5" s="21" t="n">
         <f aca="false">G5*Paramètres!$C$25</f>
         <v>20.0205315590267</v>
       </c>
@@ -5052,19 +5051,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$5</f>
         <v>6.99642231901472</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E6/(1+Paramètres!$C$6),E6)</f>
         <v>19.9166666666667</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="21" t="n">
         <f aca="false">E6*Paramètres!$C$11</f>
         <v>0.3585</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="21" t="n">
         <f aca="false">H6*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K6" s="17" t="n">
+      <c r="K6" s="30" t="n">
         <f aca="false">IF(G6=0,0,H6-G6-I6-J6)</f>
         <v>12.561744347652</v>
       </c>
@@ -5076,11 +5075,11 @@
         <f aca="false">IF(G6=0,0,E6/G6)</f>
         <v>3.41603163877703</v>
       </c>
-      <c r="N6" s="17" t="n">
+      <c r="N6" s="30" t="n">
         <f aca="false">IF(G6=0,0,K6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>7.67574434765195</v>
-      </c>
-      <c r="O6" s="22" t="n">
+        <v>12.1399110143186</v>
+      </c>
+      <c r="O6" s="21" t="n">
         <f aca="false">G6*Paramètres!$C$25</f>
         <v>20.9892669570442</v>
       </c>
@@ -5113,19 +5112,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$7</f>
         <v>4.52076519074797</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E7/(1+Paramètres!$C$6),E7)</f>
         <v>11.5833333333333</v>
       </c>
-      <c r="I7" s="22" t="n">
+      <c r="I7" s="21" t="n">
         <f aca="false">E7*Paramètres!$C$11</f>
         <v>0.2085</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="J7" s="21" t="n">
         <f aca="false">H7*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="K7" s="30" t="n">
         <f aca="false">IF(G7=0,0,H7-G7-I7-J7)</f>
         <v>6.85406814258536</v>
       </c>
@@ -5137,11 +5136,11 @@
         <f aca="false">IF(G7=0,0,E7/G7)</f>
         <v>3.07470072288807</v>
       </c>
-      <c r="N7" s="17" t="n">
+      <c r="N7" s="30" t="n">
         <f aca="false">IF(G7=0,0,K7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>1.96806814258536</v>
-      </c>
-      <c r="O7" s="22" t="n">
+        <v>6.43223480925203</v>
+      </c>
+      <c r="O7" s="21" t="n">
         <f aca="false">G7*Paramètres!$C$25</f>
         <v>13.5622955722439</v>
       </c>
@@ -5174,19 +5173,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$6</f>
         <v>3.98257885851607</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E8/(1+Paramètres!$C$6),E8)</f>
         <v>8.25</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="I8" s="21" t="n">
         <f aca="false">E8*Paramètres!$C$11</f>
         <v>0.1485</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="21" t="n">
         <f aca="false">H8*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K8" s="17" t="n">
+      <c r="K8" s="30" t="n">
         <f aca="false">IF(G8=0,0,H8-G8-I8-J8)</f>
         <v>4.11892114148393</v>
       </c>
@@ -5198,17 +5197,17 @@
         <f aca="false">IF(G8=0,0,E8/G8)</f>
         <v>2.48582648371934</v>
       </c>
-      <c r="N8" s="17" t="n">
+      <c r="N8" s="30" t="n">
         <f aca="false">IF(G8=0,0,K8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>-0.767078858516071</v>
-      </c>
-      <c r="O8" s="22" t="n">
+        <v>3.6970878081506</v>
+      </c>
+      <c r="O8" s="21" t="n">
         <f aca="false">G8*Paramètres!$C$25</f>
         <v>11.9477365755482</v>
       </c>
       <c r="P8" s="6" t="str">
         <f aca="false">IF(G8=0,"Prix fournisseur manquant",IF(N8&lt;0,"Perte si vendu seul",IF(L8&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
-        <v>Perte si vendu seul</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5235,19 +5234,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$22</f>
         <v>2.47565712826675</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E9/(1+Paramètres!$C$6),E9)</f>
         <v>16.5833333333333</v>
       </c>
-      <c r="I9" s="22" t="n">
+      <c r="I9" s="21" t="n">
         <f aca="false">E9*Paramètres!$C$11</f>
         <v>0.2985</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="J9" s="21" t="n">
         <f aca="false">H9*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="30" t="n">
         <f aca="false">IF(G9=0,0,H9-G9-I9-J9)</f>
         <v>13.8091762050666</v>
       </c>
@@ -5259,11 +5258,11 @@
         <f aca="false">IF(G9=0,0,E9/G9)</f>
         <v>8.03826982855754</v>
       </c>
-      <c r="N9" s="17" t="n">
+      <c r="N9" s="30" t="n">
         <f aca="false">IF(G9=0,0,K9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>8.92317620506659</v>
-      </c>
-      <c r="O9" s="22" t="n">
+        <v>13.3873428717333</v>
+      </c>
+      <c r="O9" s="21" t="n">
         <f aca="false">G9*Paramètres!$C$25</f>
         <v>7.42697138480024</v>
       </c>
@@ -5296,19 +5295,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$15</f>
         <v>2.47565712826675</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E10/(1+Paramètres!$C$6),E10)</f>
         <v>8.25</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="I10" s="21" t="n">
         <f aca="false">E10*Paramètres!$C$11</f>
         <v>0.1485</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="21" t="n">
         <f aca="false">H10*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="K10" s="30" t="n">
         <f aca="false">IF(G10=0,0,H10-G10-I10-J10)</f>
         <v>5.62584287173325</v>
       </c>
@@ -5320,11 +5319,11 @@
         <f aca="false">IF(G10=0,0,E10/G10)</f>
         <v>3.99893825641808</v>
       </c>
-      <c r="N10" s="17" t="n">
+      <c r="N10" s="30" t="n">
         <f aca="false">IF(G10=0,0,K10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>0.739842871733253</v>
-      </c>
-      <c r="O10" s="22" t="n">
+        <v>5.20400953839992</v>
+      </c>
+      <c r="O10" s="21" t="n">
         <f aca="false">G10*Paramètres!$C$25</f>
         <v>7.42697138480024</v>
       </c>
@@ -5357,19 +5356,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$18</f>
         <v>5.05895152297987</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H11" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E11/(1+Paramètres!$C$6),E11)</f>
         <v>10.75</v>
       </c>
-      <c r="I11" s="22" t="n">
+      <c r="I11" s="21" t="n">
         <f aca="false">E11*Paramètres!$C$11</f>
         <v>0.1935</v>
       </c>
-      <c r="J11" s="22" t="n">
+      <c r="J11" s="21" t="n">
         <f aca="false">H11*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K11" s="17" t="n">
+      <c r="K11" s="30" t="n">
         <f aca="false">IF(G11=0,0,H11-G11-I11-J11)</f>
         <v>5.49754847702013</v>
       </c>
@@ -5381,11 +5380,11 @@
         <f aca="false">IF(G11=0,0,E11/G11)</f>
         <v>2.54993548394421</v>
       </c>
-      <c r="N11" s="17" t="n">
+      <c r="N11" s="30" t="n">
         <f aca="false">IF(G11=0,0,K11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>0.611548477020127</v>
-      </c>
-      <c r="O11" s="22" t="n">
+        <v>5.07571514368679</v>
+      </c>
+      <c r="O11" s="21" t="n">
         <f aca="false">G11*Paramètres!$C$25</f>
         <v>15.1768545689396</v>
       </c>
@@ -5418,19 +5417,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$18</f>
         <v>5.05895152297987</v>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="H12" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E12/(1+Paramètres!$C$6),E12)</f>
         <v>10.75</v>
       </c>
-      <c r="I12" s="22" t="n">
+      <c r="I12" s="21" t="n">
         <f aca="false">E12*Paramètres!$C$11</f>
         <v>0.1935</v>
       </c>
-      <c r="J12" s="22" t="n">
+      <c r="J12" s="21" t="n">
         <f aca="false">H12*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K12" s="17" t="n">
+      <c r="K12" s="30" t="n">
         <f aca="false">IF(G12=0,0,H12-G12-I12-J12)</f>
         <v>5.49754847702013</v>
       </c>
@@ -5442,11 +5441,11 @@
         <f aca="false">IF(G12=0,0,E12/G12)</f>
         <v>2.54993548394421</v>
       </c>
-      <c r="N12" s="17" t="n">
+      <c r="N12" s="30" t="n">
         <f aca="false">IF(G12=0,0,K12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>0.611548477020127</v>
-      </c>
-      <c r="O12" s="22" t="n">
+        <v>5.07571514368679</v>
+      </c>
+      <c r="O12" s="21" t="n">
         <f aca="false">G12*Paramètres!$C$25</f>
         <v>15.1768545689396</v>
       </c>
@@ -5479,19 +5478,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$11</f>
         <v>2.47565712826675</v>
       </c>
-      <c r="H13" s="22" t="n">
+      <c r="H13" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E13/(1+Paramètres!$C$6),E13)</f>
         <v>5.75</v>
       </c>
-      <c r="I13" s="22" t="n">
+      <c r="I13" s="21" t="n">
         <f aca="false">E13*Paramètres!$C$11</f>
         <v>0.1035</v>
       </c>
-      <c r="J13" s="22" t="n">
+      <c r="J13" s="21" t="n">
         <f aca="false">H13*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K13" s="17" t="n">
+      <c r="K13" s="30" t="n">
         <f aca="false">IF(G13=0,0,H13-G13-I13-J13)</f>
         <v>3.17084287173326</v>
       </c>
@@ -5503,17 +5502,17 @@
         <f aca="false">IF(G13=0,0,E13/G13)</f>
         <v>2.78713878477623</v>
       </c>
-      <c r="N13" s="17" t="n">
+      <c r="N13" s="30" t="n">
         <f aca="false">IF(G13=0,0,K13-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E13&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>-1.71515712826675</v>
-      </c>
-      <c r="O13" s="22" t="n">
+        <v>2.74900953839992</v>
+      </c>
+      <c r="O13" s="21" t="n">
         <f aca="false">G13*Paramètres!$C$25</f>
         <v>7.42697138480024</v>
       </c>
       <c r="P13" s="6" t="str">
         <f aca="false">IF(G13=0,"Prix fournisseur manquant",IF(N13&lt;0,"Perte si vendu seul",IF(L13&lt;Paramètres!$C$26,"Marge faible","OK")))</f>
-        <v>Perte si vendu seul</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5540,19 +5539,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$22+'Tarifs Onsha-Sullab'!$O$18</f>
         <v>7.53460865124662</v>
       </c>
-      <c r="H14" s="22" t="n">
+      <c r="H14" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E14/(1+Paramètres!$C$6),E14)</f>
         <v>24.9166666666667</v>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="I14" s="21" t="n">
         <f aca="false">E14*Paramètres!$C$11</f>
         <v>0.4485</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="J14" s="21" t="n">
         <f aca="false">H14*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K14" s="17" t="n">
+      <c r="K14" s="30" t="n">
         <f aca="false">IF(G14=0,0,H14-G14-I14-J14)</f>
         <v>16.9335580154201</v>
       </c>
@@ -5564,11 +5563,11 @@
         <f aca="false">IF(G14=0,0,E14/G14)</f>
         <v>3.9683547459433</v>
       </c>
-      <c r="N14" s="17" t="n">
+      <c r="N14" s="30" t="n">
         <f aca="false">IF(G14=0,0,K14-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E14&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>12.0475580154201</v>
-      </c>
-      <c r="O14" s="22" t="n">
+        <v>16.5117246820867</v>
+      </c>
+      <c r="O14" s="21" t="n">
         <f aca="false">G14*Paramètres!$C$25</f>
         <v>22.6038259537399</v>
       </c>
@@ -5601,19 +5600,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$16+'Tarifs Onsha-Sullab'!$O$22+'Tarifs Onsha-Sullab'!$O$18</f>
         <v>14.2081191709222</v>
       </c>
-      <c r="H15" s="22" t="n">
+      <c r="H15" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E15/(1+Paramètres!$C$6),E15)</f>
         <v>41.5833333333333</v>
       </c>
-      <c r="I15" s="22" t="n">
+      <c r="I15" s="21" t="n">
         <f aca="false">E15*Paramètres!$C$11</f>
         <v>0.7485</v>
       </c>
-      <c r="J15" s="22" t="n">
+      <c r="J15" s="21" t="n">
         <f aca="false">H15*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K15" s="17" t="n">
+      <c r="K15" s="30" t="n">
         <f aca="false">IF(G15=0,0,H15-G15-I15-J15)</f>
         <v>26.6267141624111</v>
       </c>
@@ -5625,11 +5624,11 @@
         <f aca="false">IF(G15=0,0,E15/G15)</f>
         <v>3.51207639798823</v>
       </c>
-      <c r="N15" s="17" t="n">
+      <c r="N15" s="30" t="n">
         <f aca="false">IF(G15=0,0,K15-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E15&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>21.7407141624111</v>
-      </c>
-      <c r="O15" s="22" t="n">
+        <v>26.2048808290778</v>
+      </c>
+      <c r="O15" s="21" t="n">
         <f aca="false">G15*Paramètres!$C$25</f>
         <v>42.6243575127666</v>
       </c>
@@ -5662,19 +5661,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$17</f>
         <v>21.5274532892761</v>
       </c>
-      <c r="H16" s="22" t="n">
+      <c r="H16" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E16/(1+Paramètres!$C$6),E16)</f>
         <v>49.9166666666667</v>
       </c>
-      <c r="I16" s="22" t="n">
+      <c r="I16" s="21" t="n">
         <f aca="false">E16*Paramètres!$C$11</f>
         <v>0.8985</v>
       </c>
-      <c r="J16" s="22" t="n">
+      <c r="J16" s="21" t="n">
         <f aca="false">H16*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K16" s="17" t="n">
+      <c r="K16" s="30" t="n">
         <f aca="false">IF(G16=0,0,H16-G16-I16-J16)</f>
         <v>27.4907133773906</v>
       </c>
@@ -5686,11 +5685,11 @@
         <f aca="false">IF(G16=0,0,E16/G16)</f>
         <v>2.78249355346827</v>
       </c>
-      <c r="N16" s="17" t="n">
+      <c r="N16" s="30" t="n">
         <f aca="false">IF(G16=0,0,K16-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E16&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>22.6047133773906</v>
-      </c>
-      <c r="O16" s="22" t="n">
+        <v>27.0688800440573</v>
+      </c>
+      <c r="O16" s="21" t="n">
         <f aca="false">G16*Paramètres!$C$25</f>
         <v>64.5823598678282</v>
       </c>
@@ -5723,19 +5722,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$10</f>
         <v>10.9790011775308</v>
       </c>
-      <c r="H17" s="22" t="n">
+      <c r="H17" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E17/(1+Paramètres!$C$6),E17)</f>
         <v>24.9166666666667</v>
       </c>
-      <c r="I17" s="22" t="n">
+      <c r="I17" s="21" t="n">
         <f aca="false">E17*Paramètres!$C$11</f>
         <v>0.4485</v>
       </c>
-      <c r="J17" s="22" t="n">
+      <c r="J17" s="21" t="n">
         <f aca="false">H17*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K17" s="17" t="n">
+      <c r="K17" s="30" t="n">
         <f aca="false">IF(G17=0,0,H17-G17-I17-J17)</f>
         <v>13.4891654891359</v>
       </c>
@@ -5747,11 +5746,11 @@
         <f aca="false">IF(G17=0,0,E17/G17)</f>
         <v>2.72338070800031</v>
       </c>
-      <c r="N17" s="17" t="n">
+      <c r="N17" s="30" t="n">
         <f aca="false">IF(G17=0,0,K17-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E17&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>8.60316548913588</v>
-      </c>
-      <c r="O17" s="22" t="n">
+        <v>13.0673321558026</v>
+      </c>
+      <c r="O17" s="21" t="n">
         <f aca="false">G17*Paramètres!$C$25</f>
         <v>32.9370035325924</v>
       </c>
@@ -5784,19 +5783,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$16+'Tarifs Onsha-Sullab'!$O$17</f>
         <v>28.2009638089516</v>
       </c>
-      <c r="H18" s="22" t="n">
+      <c r="H18" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E18/(1+Paramètres!$C$6),E18)</f>
         <v>66.5833333333333</v>
       </c>
-      <c r="I18" s="22" t="n">
+      <c r="I18" s="21" t="n">
         <f aca="false">E18*Paramètres!$C$11</f>
         <v>1.1985</v>
       </c>
-      <c r="J18" s="22" t="n">
+      <c r="J18" s="21" t="n">
         <f aca="false">H18*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K18" s="17" t="n">
+      <c r="K18" s="30" t="n">
         <f aca="false">IF(G18=0,0,H18-G18-I18-J18)</f>
         <v>37.1838695243817</v>
       </c>
@@ -5808,11 +5807,11 @@
         <f aca="false">IF(G18=0,0,E18/G18)</f>
         <v>2.83323650004607</v>
       </c>
-      <c r="N18" s="17" t="n">
+      <c r="N18" s="30" t="n">
         <f aca="false">IF(G18=0,0,K18-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E18&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>32.2978695243817</v>
-      </c>
-      <c r="O18" s="22" t="n">
+        <v>36.7620361910484</v>
+      </c>
+      <c r="O18" s="21" t="n">
         <f aca="false">G18*Paramètres!$C$25</f>
         <v>84.6028914268549</v>
       </c>
@@ -5845,19 +5844,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$5+'Tarifs Onsha-Sullab'!$O$7+'Tarifs Onsha-Sullab'!$O$10</f>
         <v>22.4961886872935</v>
       </c>
-      <c r="H19" s="22" t="n">
+      <c r="H19" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E19/(1+Paramètres!$C$6),E19)</f>
         <v>49.9166666666667</v>
       </c>
-      <c r="I19" s="22" t="n">
+      <c r="I19" s="21" t="n">
         <f aca="false">E19*Paramètres!$C$11</f>
         <v>0.8985</v>
       </c>
-      <c r="J19" s="22" t="n">
+      <c r="J19" s="21" t="n">
         <f aca="false">H19*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K19" s="17" t="n">
+      <c r="K19" s="30" t="n">
         <f aca="false">IF(G19=0,0,H19-G19-I19-J19)</f>
         <v>26.5219779793732</v>
       </c>
@@ -5869,11 +5868,11 @@
         <f aca="false">IF(G19=0,0,E19/G19)</f>
         <v>2.66267325690744</v>
       </c>
-      <c r="N19" s="17" t="n">
+      <c r="N19" s="30" t="n">
         <f aca="false">IF(G19=0,0,K19-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E19&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>21.6359779793732</v>
-      </c>
-      <c r="O19" s="22" t="n">
+        <v>26.1001446460399</v>
+      </c>
+      <c r="O19" s="21" t="n">
         <f aca="false">G19*Paramètres!$C$25</f>
         <v>67.4885660618804</v>
       </c>
@@ -5906,19 +5905,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$23</f>
         <v>5.81241238810454</v>
       </c>
-      <c r="H20" s="22" t="n">
+      <c r="H20" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E20/(1+Paramètres!$C$6),E20)</f>
         <v>21.5833333333333</v>
       </c>
-      <c r="I20" s="22" t="n">
+      <c r="I20" s="21" t="n">
         <f aca="false">E20*Paramètres!$C$11</f>
         <v>0.3885</v>
       </c>
-      <c r="J20" s="22" t="n">
+      <c r="J20" s="21" t="n">
         <f aca="false">H20*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K20" s="17" t="n">
+      <c r="K20" s="30" t="n">
         <f aca="false">IF(G20=0,0,H20-G20-I20-J20)</f>
         <v>15.3824209452288</v>
       </c>
@@ -5930,11 +5929,11 @@
         <f aca="false">IF(G20=0,0,E20/G20)</f>
         <v>4.455981143562</v>
       </c>
-      <c r="N20" s="17" t="n">
+      <c r="N20" s="30" t="n">
         <f aca="false">IF(G20=0,0,K20-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E20&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>10.4964209452288</v>
-      </c>
-      <c r="O20" s="22" t="n">
+        <v>14.9605876118955</v>
+      </c>
+      <c r="O20" s="21" t="n">
         <f aca="false">G20*Paramètres!$C$25</f>
         <v>17.4372371643136</v>
       </c>
@@ -5967,19 +5966,19 @@
         <f aca="false">'Tarifs Onsha-Sullab'!$O$24</f>
         <v>2.47565712826675</v>
       </c>
-      <c r="H21" s="22" t="n">
+      <c r="H21" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E21/(1+Paramètres!$C$6),E21)</f>
         <v>9.91666666666667</v>
       </c>
-      <c r="I21" s="22" t="n">
+      <c r="I21" s="21" t="n">
         <f aca="false">E21*Paramètres!$C$11</f>
         <v>0.1785</v>
       </c>
-      <c r="J21" s="22" t="n">
+      <c r="J21" s="21" t="n">
         <f aca="false">H21*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K21" s="17" t="n">
+      <c r="K21" s="30" t="n">
         <f aca="false">IF(G21=0,0,H21-G21-I21-J21)</f>
         <v>7.26250953839992</v>
       </c>
@@ -5991,11 +5990,11 @@
         <f aca="false">IF(G21=0,0,E21/G21)</f>
         <v>4.80680457084597</v>
       </c>
-      <c r="N21" s="17" t="n">
+      <c r="N21" s="30" t="n">
         <f aca="false">IF(G21=0,0,K21-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E21&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>2.37650953839992</v>
-      </c>
-      <c r="O21" s="22" t="n">
+        <v>6.84067620506659</v>
+      </c>
+      <c r="O21" s="21" t="n">
         <f aca="false">G21*Paramètres!$C$25</f>
         <v>7.42697138480024</v>
       </c>
@@ -6028,19 +6027,19 @@
         <f aca="false">'Tarifs Shift'!$L$5+1/6*'Tarifs Shift'!$L$8</f>
         <v>15.4817177242888</v>
       </c>
-      <c r="H22" s="22" t="n">
+      <c r="H22" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E22/(1+Paramètres!$C$6),E22)</f>
         <v>49.9166666666667</v>
       </c>
-      <c r="I22" s="22" t="n">
+      <c r="I22" s="21" t="n">
         <f aca="false">E22*Paramètres!$C$11</f>
         <v>0.8985</v>
       </c>
-      <c r="J22" s="22" t="n">
+      <c r="J22" s="21" t="n">
         <f aca="false">H22*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K22" s="17" t="n">
+      <c r="K22" s="30" t="n">
         <f aca="false">IF(G22=0,0,H22-G22-I22-J22)</f>
         <v>33.5364489423778</v>
       </c>
@@ -6052,11 +6051,11 @@
         <f aca="false">IF(G22=0,0,E22/G22)</f>
         <v>3.86907971497404</v>
       </c>
-      <c r="N22" s="17" t="n">
+      <c r="N22" s="30" t="n">
         <f aca="false">IF(G22=0,0,K22-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E22&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>28.6504489423778</v>
-      </c>
-      <c r="O22" s="22" t="n">
+        <v>33.1146156090445</v>
+      </c>
+      <c r="O22" s="21" t="n">
         <f aca="false">G22*Paramètres!$C$25</f>
         <v>46.4451531728665</v>
       </c>
@@ -6089,19 +6088,19 @@
         <f aca="false">'Tarifs Shift'!$L$7</f>
         <v>34.771772428884</v>
       </c>
-      <c r="H23" s="22" t="n">
+      <c r="H23" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E23/(1+Paramètres!$C$6),E23)</f>
         <v>91.5833333333333</v>
       </c>
-      <c r="I23" s="22" t="n">
+      <c r="I23" s="21" t="n">
         <f aca="false">E23*Paramètres!$C$11</f>
         <v>1.6485</v>
       </c>
-      <c r="J23" s="22" t="n">
+      <c r="J23" s="21" t="n">
         <f aca="false">H23*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K23" s="17" t="n">
+      <c r="K23" s="30" t="n">
         <f aca="false">IF(G23=0,0,H23-G23-I23-J23)</f>
         <v>55.1630609044493</v>
       </c>
@@ -6113,11 +6112,11 @@
         <f aca="false">IF(G23=0,0,E23/G23)</f>
         <v>3.16060966477248</v>
       </c>
-      <c r="N23" s="17" t="n">
+      <c r="N23" s="30" t="n">
         <f aca="false">IF(G23=0,0,K23-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E23&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>46.267227571116</v>
-      </c>
-      <c r="O23" s="22" t="n">
+        <v>49.9130609044493</v>
+      </c>
+      <c r="O23" s="21" t="n">
         <f aca="false">G23*Paramètres!$C$25</f>
         <v>104.315317286652</v>
       </c>
@@ -6150,19 +6149,19 @@
         <f aca="false">'Tarifs Shift'!$L$9</f>
         <v>5.46413566739606</v>
       </c>
-      <c r="H24" s="22" t="n">
+      <c r="H24" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E24/(1+Paramètres!$C$6),E24)</f>
         <v>21.5833333333333</v>
       </c>
-      <c r="I24" s="22" t="n">
+      <c r="I24" s="21" t="n">
         <f aca="false">E24*Paramètres!$C$11</f>
         <v>0.3885</v>
       </c>
-      <c r="J24" s="22" t="n">
+      <c r="J24" s="21" t="n">
         <f aca="false">H24*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K24" s="17" t="n">
+      <c r="K24" s="30" t="n">
         <f aca="false">IF(G24=0,0,H24-G24-I24-J24)</f>
         <v>15.7306976659373</v>
       </c>
@@ -6174,11 +6173,11 @@
         <f aca="false">IF(G24=0,0,E24/G24)</f>
         <v>4.73999943935189</v>
       </c>
-      <c r="N24" s="17" t="n">
+      <c r="N24" s="30" t="n">
         <f aca="false">IF(G24=0,0,K24-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E24&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>10.8446976659373</v>
-      </c>
-      <c r="O24" s="22" t="n">
+        <v>15.3088643326039</v>
+      </c>
+      <c r="O24" s="21" t="n">
         <f aca="false">G24*Paramètres!$C$25</f>
         <v>16.3924070021882</v>
       </c>
@@ -6211,19 +6210,19 @@
         <f aca="false">'Tarifs Shift'!$L$8</f>
         <v>6.45761487964989</v>
       </c>
-      <c r="H25" s="22" t="n">
+      <c r="H25" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),E25/(1+Paramètres!$C$6),E25)</f>
         <v>27.4166666666667</v>
       </c>
-      <c r="I25" s="22" t="n">
+      <c r="I25" s="21" t="n">
         <f aca="false">E25*Paramètres!$C$11</f>
         <v>0.4935</v>
       </c>
-      <c r="J25" s="22" t="n">
+      <c r="J25" s="21" t="n">
         <f aca="false">H25*Paramètres!$C$13</f>
         <v>0</v>
       </c>
-      <c r="K25" s="17" t="n">
+      <c r="K25" s="30" t="n">
         <f aca="false">IF(G25=0,0,H25-G25-I25-J25)</f>
         <v>20.4655517870168</v>
       </c>
@@ -6235,11 +6234,11 @@
         <f aca="false">IF(G25=0,0,E25/G25)</f>
         <v>5.09476031215162</v>
       </c>
-      <c r="N25" s="17" t="n">
+      <c r="N25" s="30" t="n">
         <f aca="false">IF(G25=0,0,K25-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E25&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>15.5795517870168</v>
-      </c>
-      <c r="O25" s="22" t="n">
+        <v>20.0437184536834</v>
+      </c>
+      <c r="O25" s="21" t="n">
         <f aca="false">G25*Paramètres!$C$25</f>
         <v>19.3728446389497</v>
       </c>
@@ -6288,7 +6287,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>310</v>
       </c>
     </row>
@@ -6390,7 +6389,7 @@
       <c r="B13" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="D13" s="22" t="n">
+      <c r="D13" s="21" t="n">
         <f aca="false">SUM(D6:D11)</f>
         <v>75.7</v>
       </c>
@@ -6402,9 +6401,9 @@
       <c r="B14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="21" t="n">
         <f aca="false">IF(OR(D13=0,D13&gt;=Paramètres!$C$16),0,Paramètres!$C$15)</f>
-        <v>4.9</v>
+        <v>5.9</v>
       </c>
       <c r="F14" s="32"/>
     </row>
@@ -6412,9 +6411,9 @@
       <c r="B15" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="D15" s="22" t="n">
+      <c r="D15" s="21" t="n">
         <f aca="false">IF((Paramètres!$C$5="Assujettie"),(D13+D14)/(1+Paramètres!$C$6),D13+D14)</f>
-        <v>67.1666666666667</v>
+        <v>68</v>
       </c>
       <c r="F15" s="32"/>
     </row>
@@ -6422,7 +6421,7 @@
       <c r="B16" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="D16" s="21" t="n">
         <f aca="false">-SUM(E6:E11)</f>
         <v>-24.3260222168819</v>
       </c>
@@ -6432,9 +6431,9 @@
       <c r="B17" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="D17" s="22" t="n">
+      <c r="D17" s="21" t="n">
         <f aca="false">IF(D13=0,0,-((D13+D14)*Paramètres!$C$11+Paramètres!$C$12))</f>
-        <v>-1.459</v>
+        <v>-1.474</v>
       </c>
       <c r="F17" s="32"/>
     </row>
@@ -6442,7 +6441,7 @@
       <c r="B18" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="D18" s="22" t="n">
+      <c r="D18" s="21" t="n">
         <f aca="false">-D15*Paramètres!$C$13</f>
         <v>-0</v>
       </c>
@@ -6451,36 +6450,36 @@
       <c r="B19" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="D19" s="22" t="n">
+      <c r="D19" s="21" t="n">
         <f aca="false">IF(D13=0,0,-Paramètres!$C$14*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1))</f>
-        <v>-4.58333333333333</v>
+        <v>-3.33333333333333</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="D20" s="22" t="n">
+      <c r="D20" s="21" t="n">
         <f aca="false">IF(D13=0,0,-(Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1))</f>
-        <v>-4.0625</v>
+        <v>-1.66666666666667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="D21" s="22" t="n">
+      <c r="D21" s="21" t="n">
         <f aca="false">IF(D13=0,0,-Paramètres!$C$24)</f>
         <v>-0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="24" t="s">
         <v>322</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="30" t="n">
         <f aca="false">SUM(D15:D21)</f>
-        <v>32.7358111164514</v>
+        <v>37.1999777831181</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6489,7 +6488,7 @@
       </c>
       <c r="D23" s="36" t="n">
         <f aca="false">IF(D15=0,0,D22/D15)</f>
-        <v>0.487381803222601</v>
+        <v>0.54705849681056</v>
       </c>
     </row>
   </sheetData>
@@ -6532,7 +6531,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>325</v>
       </c>
     </row>
@@ -6639,28 +6638,28 @@
       <c r="D14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="24" t="s">
         <v>341</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="30" t="n">
         <f aca="false">SUM(C6:C14)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)</f>
         <v>22.0833333333333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="24" t="s">
         <v>342</v>
       </c>
       <c r="C17" s="35" t="n">
         <f aca="false">'Simulateur commande'!D22</f>
-        <v>32.7358111164514</v>
+        <v>37.1999777831181</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="24" t="s">
         <v>344</v>
       </c>
       <c r="C18" s="39" t="n">

</xml_diff>

<commit_message>
Gestion : livraison offerte dès 80 € (France)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6qThdJp8fvnL986bvjdNe
</commit_message>
<xml_diff>
--- a/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
+++ b/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
@@ -175,7 +175,7 @@
     <t xml:space="preserve">Livraison offerte à partir de (TTC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Repris de tes tarifs Shopify (livraison gratuite dès 100 € d'achat).</t>
+    <t xml:space="preserve">France : livraison offerte dès 80 €, non cumulable avec les remises (sauf code exceptionnel). Dès 100 € après remise dans tous les cas.</t>
   </si>
   <si>
     <t xml:space="preserve">Emballage : prix d'un lot de cartons (TTC)</t>
@@ -2612,7 +2612,7 @@
         <v>47</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
Gestion : coût étiquette réel Boxtal (3,07 € HT)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6qThdJp8fvnL986bvjdNe
</commit_message>
<xml_diff>
--- a/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
+++ b/sunsoari-theme/gestion/Sunsoari_Marges.xlsx
@@ -163,7 +163,7 @@
     <t xml:space="preserve">Ce que TU paies au transporteur par colis (TTC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Coût moyen réel d'une étiquette Mondial Relay / Colissimo pour un colis de moins de 1 kg. Exemple : remplace-le par le montant de tes factures transporteur.</t>
+    <t xml:space="preserve">Boxtal, octobre 2026 : Mondial Relay 3,07 € HT (500 g, sans assurance), Chrono 2Shop Direct 3,10 € HT, soit environ 3,70 € TTC.</t>
   </si>
   <si>
     <t xml:space="preserve">Livraison payée par la cliente (TTC)</t>
@@ -2023,11 +2023,11 @@
       </c>
       <c r="K5" s="30" t="n">
         <f aca="false">I5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>9.01843028737359</v>
+        <v>9.26843028737359</v>
       </c>
       <c r="L5" s="35" t="n">
         <f aca="false">'Marges produits'!$N$11</f>
-        <v>5.07571514368679</v>
+        <v>5.32571514368679</v>
       </c>
       <c r="M5" s="6" t="str">
         <f aca="false">IF(E5&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2073,11 +2073,11 @@
       </c>
       <c r="K6" s="30" t="n">
         <f aca="false">I6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>16.0855272414138</v>
+        <v>16.3355272414138</v>
       </c>
       <c r="L6" s="35" t="n">
         <f aca="false">'Marges produits'!$N$11</f>
-        <v>5.07571514368679</v>
+        <v>5.32571514368679</v>
       </c>
       <c r="M6" s="6" t="str">
         <f aca="false">IF(E6&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2123,11 +2123,11 @@
       </c>
       <c r="K7" s="30" t="n">
         <f aca="false">I7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>6.7993619485331</v>
+        <v>7.0493619485331</v>
       </c>
       <c r="L7" s="35" t="n">
         <f aca="false">'Marges produits'!$N$13</f>
-        <v>2.74900953839992</v>
+        <v>2.99900953839992</v>
       </c>
       <c r="M7" s="6" t="str">
         <f aca="false">IF(E7&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2173,11 +2173,11 @@
       </c>
       <c r="K8" s="30" t="n">
         <f aca="false">I8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>13.2840572303995</v>
+        <v>13.5340572303995</v>
       </c>
       <c r="L8" s="35" t="n">
         <f aca="false">'Marges produits'!$N$13</f>
-        <v>2.74900953839992</v>
+        <v>2.99900953839992</v>
       </c>
       <c r="M8" s="6" t="str">
         <f aca="false">IF(E8&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2223,11 +2223,11 @@
       </c>
       <c r="K9" s="30" t="n">
         <f aca="false">I9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>13.0673321558025</v>
+        <v>13.3173321558025</v>
       </c>
       <c r="L9" s="35" t="n">
         <f aca="false">'Marges produits'!$N$8</f>
-        <v>3.6970878081506</v>
+        <v>3.9470878081506</v>
       </c>
       <c r="M9" s="6" t="str">
         <f aca="false">IF(E9&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2273,11 +2273,11 @@
       </c>
       <c r="K10" s="30" t="n">
         <f aca="false">I10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>10.9131362851707</v>
+        <v>11.1631362851707</v>
       </c>
       <c r="L10" s="35" t="n">
         <f aca="false">'Marges produits'!$N$7</f>
-        <v>6.43223480925203</v>
+        <v>6.68223480925203</v>
       </c>
       <c r="M10" s="6" t="str">
         <f aca="false">IF(E10&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2323,11 +2323,11 @@
       </c>
       <c r="K11" s="30" t="n">
         <f aca="false">I11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>29.2259769980975</v>
+        <v>29.4759769980975</v>
       </c>
       <c r="L11" s="35" t="n">
         <f aca="false">'Marges produits'!$N$16</f>
-        <v>27.0688800440573</v>
+        <v>27.3188800440573</v>
       </c>
       <c r="M11" s="6" t="str">
         <f aca="false">IF(E11&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2373,11 +2373,11 @@
       </c>
       <c r="K12" s="30" t="n">
         <f aca="false">I12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11)</f>
-        <v>17.9153607710023</v>
+        <v>18.1653607710023</v>
       </c>
       <c r="L12" s="35" t="n">
         <f aca="false">'Marges produits'!$N$17</f>
-        <v>13.0673321558026</v>
+        <v>13.3173321558026</v>
       </c>
       <c r="M12" s="6" t="str">
         <f aca="false">IF(E12&gt;=Paramètres!$C$16,"Oui","Non")</f>
@@ -2589,8 +2589,8 @@
       <c r="B14" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>4</v>
+      <c r="C14" s="14" t="n">
+        <v>3.7</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>44</v>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="N5" s="30" t="n">
         <f aca="false">IF(G5=0,0,K5-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E5&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>12.4628228136578</v>
+        <v>12.7128228136578</v>
       </c>
       <c r="O5" s="21" t="n">
         <f aca="false">G5*Paramètres!$C$25</f>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="N6" s="30" t="n">
         <f aca="false">IF(G6=0,0,K6-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E6&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>12.1399110143186</v>
+        <v>12.3899110143186</v>
       </c>
       <c r="O6" s="21" t="n">
         <f aca="false">G6*Paramètres!$C$25</f>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="N7" s="30" t="n">
         <f aca="false">IF(G7=0,0,K7-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E7&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>6.43223480925203</v>
+        <v>6.68223480925203</v>
       </c>
       <c r="O7" s="21" t="n">
         <f aca="false">G7*Paramètres!$C$25</f>
@@ -5199,7 +5199,7 @@
       </c>
       <c r="N8" s="30" t="n">
         <f aca="false">IF(G8=0,0,K8-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E8&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>3.6970878081506</v>
+        <v>3.9470878081506</v>
       </c>
       <c r="O8" s="21" t="n">
         <f aca="false">G8*Paramètres!$C$25</f>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="N9" s="30" t="n">
         <f aca="false">IF(G9=0,0,K9-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E9&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>13.3873428717333</v>
+        <v>13.6373428717333</v>
       </c>
       <c r="O9" s="21" t="n">
         <f aca="false">G9*Paramètres!$C$25</f>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="N10" s="30" t="n">
         <f aca="false">IF(G10=0,0,K10-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E10&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>5.20400953839992</v>
+        <v>5.45400953839992</v>
       </c>
       <c r="O10" s="21" t="n">
         <f aca="false">G10*Paramètres!$C$25</f>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="N11" s="30" t="n">
         <f aca="false">IF(G11=0,0,K11-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E11&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>5.07571514368679</v>
+        <v>5.32571514368679</v>
       </c>
       <c r="O11" s="21" t="n">
         <f aca="false">G11*Paramètres!$C$25</f>
@@ -5443,7 +5443,7 @@
       </c>
       <c r="N12" s="30" t="n">
         <f aca="false">IF(G12=0,0,K12-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E12&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>5.07571514368679</v>
+        <v>5.32571514368679</v>
       </c>
       <c r="O12" s="21" t="n">
         <f aca="false">G12*Paramètres!$C$25</f>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="N13" s="30" t="n">
         <f aca="false">IF(G13=0,0,K13-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E13&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>2.74900953839992</v>
+        <v>2.99900953839992</v>
       </c>
       <c r="O13" s="21" t="n">
         <f aca="false">G13*Paramètres!$C$25</f>
@@ -5565,7 +5565,7 @@
       </c>
       <c r="N14" s="30" t="n">
         <f aca="false">IF(G14=0,0,K14-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E14&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>16.5117246820867</v>
+        <v>16.7617246820867</v>
       </c>
       <c r="O14" s="21" t="n">
         <f aca="false">G14*Paramètres!$C$25</f>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="N15" s="30" t="n">
         <f aca="false">IF(G15=0,0,K15-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E15&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>26.2048808290778</v>
+        <v>26.4548808290778</v>
       </c>
       <c r="O15" s="21" t="n">
         <f aca="false">G15*Paramètres!$C$25</f>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="N16" s="30" t="n">
         <f aca="false">IF(G16=0,0,K16-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E16&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>27.0688800440573</v>
+        <v>27.3188800440573</v>
       </c>
       <c r="O16" s="21" t="n">
         <f aca="false">G16*Paramètres!$C$25</f>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="N17" s="30" t="n">
         <f aca="false">IF(G17=0,0,K17-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E17&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>13.0673321558026</v>
+        <v>13.3173321558026</v>
       </c>
       <c r="O17" s="21" t="n">
         <f aca="false">G17*Paramètres!$C$25</f>
@@ -5809,7 +5809,7 @@
       </c>
       <c r="N18" s="30" t="n">
         <f aca="false">IF(G18=0,0,K18-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E18&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>36.7620361910484</v>
+        <v>37.0120361910484</v>
       </c>
       <c r="O18" s="21" t="n">
         <f aca="false">G18*Paramètres!$C$25</f>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="N19" s="30" t="n">
         <f aca="false">IF(G19=0,0,K19-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E19&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>26.1001446460399</v>
+        <v>26.3501446460399</v>
       </c>
       <c r="O19" s="21" t="n">
         <f aca="false">G19*Paramètres!$C$25</f>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="N20" s="30" t="n">
         <f aca="false">IF(G20=0,0,K20-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E20&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>14.9605876118955</v>
+        <v>15.2105876118955</v>
       </c>
       <c r="O20" s="21" t="n">
         <f aca="false">G20*Paramètres!$C$25</f>
@@ -5992,7 +5992,7 @@
       </c>
       <c r="N21" s="30" t="n">
         <f aca="false">IF(G21=0,0,K21-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E21&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>6.84067620506659</v>
+        <v>7.09067620506659</v>
       </c>
       <c r="O21" s="21" t="n">
         <f aca="false">G21*Paramètres!$C$25</f>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="N22" s="30" t="n">
         <f aca="false">IF(G22=0,0,K22-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E22&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>33.1146156090445</v>
+        <v>33.3646156090445</v>
       </c>
       <c r="O22" s="21" t="n">
         <f aca="false">G22*Paramètres!$C$25</f>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="N23" s="30" t="n">
         <f aca="false">IF(G23=0,0,K23-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E23&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>49.9130609044493</v>
+        <v>50.1630609044493</v>
       </c>
       <c r="O23" s="21" t="n">
         <f aca="false">G23*Paramètres!$C$25</f>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="N24" s="30" t="n">
         <f aca="false">IF(G24=0,0,K24-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E24&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>15.3088643326039</v>
+        <v>15.5588643326039</v>
       </c>
       <c r="O24" s="21" t="n">
         <f aca="false">G24*Paramètres!$C$25</f>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="N25" s="30" t="n">
         <f aca="false">IF(G25=0,0,K25-Paramètres!$C$12-(Paramètres!$C$14+Paramètres!$C$22+Paramètres!$C$23)*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)-Paramètres!$C$24+IF(E25&gt;=Paramètres!$C$16,0,Paramètres!$C$15*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1)*(1-Paramètres!$C$13)-Paramètres!$C$15*Paramètres!$C$11))</f>
-        <v>20.0437184536834</v>
+        <v>20.2937184536834</v>
       </c>
       <c r="O25" s="21" t="n">
         <f aca="false">G25*Paramètres!$C$25</f>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="D19" s="21" t="n">
         <f aca="false">IF(D13=0,0,-Paramètres!$C$14*IF((Paramètres!$C$5="Assujettie"),1/(1+Paramètres!$C$6),1))</f>
-        <v>-3.33333333333333</v>
+        <v>-3.08333333333333</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="D22" s="30" t="n">
         <f aca="false">SUM(D15:D21)</f>
-        <v>37.1999777831181</v>
+        <v>37.4499777831181</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6488,7 +6488,7 @@
       </c>
       <c r="D23" s="36" t="n">
         <f aca="false">IF(D15=0,0,D22/D15)</f>
-        <v>0.54705849681056</v>
+        <v>0.550734967398795</v>
       </c>
     </row>
   </sheetData>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="C17" s="35" t="n">
         <f aca="false">'Simulateur commande'!D22</f>
-        <v>37.1999777831181</v>
+        <v>37.4499777831181</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>343</v>

</xml_diff>